<commit_message>
Update prediction workflow and add evaluation/ausrap modules
</commit_message>
<xml_diff>
--- a/data/templates/prediction_output_template.xlsx
+++ b/data/templates/prediction_output_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R76c29b47516544f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction_Output" sheetId="2" r:id="R250720a06dae4297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="3" r:id="R76a8ade15169442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Re7ca18a805254ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction_Output" sheetId="2" r:id="R7a9fc057e75c4cc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="3" r:id="Rad88a77b8a1c46a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,13 +22,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="0" formatCode="General"/>
     <x:numFmt numFmtId="59" formatCode="0.000000"/>
     <x:numFmt numFmtId="60" formatCode="0.000"/>
     <x:numFmt numFmtId="61" formatCode="0.0"/>
+    <x:numFmt numFmtId="200" formatCode="0.00"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:color indexed="8"/>
@@ -62,6 +64,17 @@
       <x:color rgb="FF000000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color indexed="8"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color indexed="8"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -76,7 +89,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="8">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -162,13 +175,27 @@
         <x:color rgb="FF333333"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment vertical="bottom"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="bottom"/>
     </x:xf>
@@ -243,6 +270,57 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -515,15 +593,15 @@
       <x:c r="D5" s="9"/>
       <x:c r="E5" s="10"/>
     </x:row>
-    <x:row r="6" ht="13.550000190734863" customHeight="1">
+    <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>Result scope</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>The formal result contains only predicted pedestrian counts; observed and RAP data are separate evaluation sources.</x:v>
-      </x:c>
-      <x:c r="C6" s="9"/>
-      <x:c r="D6" s="9"/>
+      <x:c r="B6" s="21" t="str">
+        <x:v>Model predictions with existing AusRAP categories, derived intervals and client-recoded estimates. Accuracy metrics are not computed.</x:v>
+      </x:c>
+      <x:c r="C6" s="41"/>
+      <x:c r="D6" s="41"/>
       <x:c r="E6" s="10"/>
     </x:row>
     <x:row r="7" ht="13.550000190734863" customHeight="1">
@@ -570,15 +648,15 @@
       <x:c r="D10" s="9"/>
       <x:c r="E10" s="10"/>
     </x:row>
-    <x:row r="11" ht="13.550000190734863" customHeight="1">
+    <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="7" t="str">
         <x:v>Statuses</x:v>
       </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>Read location_status, status and message for road matching and prediction outcomes.</x:v>
-      </x:c>
-      <x:c r="C11" s="9"/>
-      <x:c r="D11" s="9"/>
+      <x:c r="B11" s="21" t="str">
+        <x:v>Read location_status for location matching, status/message for prediction, and comparison_status/comparison_notes for AusRAP reference availability.</x:v>
+      </x:c>
+      <x:c r="C11" s="41"/>
+      <x:c r="D11" s="41"/>
       <x:c r="E11" s="10"/>
     </x:row>
     <x:row r="12" ht="13.550000190734863" customHeight="1">
@@ -608,7 +686,7 @@
         <x:v>Schema version</x:v>
       </x:c>
       <x:c r="B14" s="8" t="str">
-        <x:v>prediction_output_v4</x:v>
+        <x:v>prediction_output_v5</x:v>
       </x:c>
       <x:c r="C14" s="9"/>
       <x:c r="D14" s="9"/>
@@ -645,321 +723,537 @@
         <x:v>Type</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-      <x:c r="D18" s="12"/>
+        <x:v>English label / meaning</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>中文含义</x:v>
+      </x:c>
       <x:c r="E18" s="10"/>
     </x:row>
-    <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="8" t="str">
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" s="21" t="str">
         <x:v>site_id</x:v>
       </x:c>
-      <x:c r="B19" s="8" t="str">
+      <x:c r="B19" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C19" s="21" t="str">
         <x:v>Unique input location ID</x:v>
       </x:c>
-      <x:c r="D19" s="8"/>
+      <x:c r="D19" s="21" t="str">
+        <x:v>站点编号</x:v>
+      </x:c>
       <x:c r="E19" s="10"/>
     </x:row>
-    <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="8" t="str">
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" s="21" t="str">
         <x:v>input_type</x:v>
       </x:c>
-      <x:c r="B20" s="8" t="str">
+      <x:c r="B20" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C20" s="21" t="str">
         <x:v>Coordinates, road_slk, road_segment or both</x:v>
       </x:c>
-      <x:c r="D20" s="8"/>
+      <x:c r="D20" s="21" t="str">
+        <x:v>输入类型</x:v>
+      </x:c>
       <x:c r="E20" s="10"/>
     </x:row>
-    <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="8" t="str">
+    <x:row r="21" ht="54" customHeight="1">
+      <x:c r="A21" s="21" t="str">
         <x:v>road_no</x:v>
       </x:c>
-      <x:c r="B21" s="8" t="str">
+      <x:c r="B21" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C21" s="21" t="str">
         <x:v>Supplied official road number</x:v>
       </x:c>
-      <x:c r="D21" s="8"/>
+      <x:c r="D21" s="21" t="str">
+        <x:v>输入道路编号</x:v>
+      </x:c>
       <x:c r="E21" s="10"/>
     </x:row>
-    <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="8" t="str">
+    <x:row r="22" ht="54" customHeight="1">
+      <x:c r="A22" s="21" t="str">
         <x:v>slk_km</x:v>
       </x:c>
-      <x:c r="B22" s="8" t="str">
+      <x:c r="B22" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C22" s="21" t="str">
         <x:v>Supplied point SLK in kilometres</x:v>
       </x:c>
-      <x:c r="D22" s="8"/>
+      <x:c r="D22" s="21" t="str">
+        <x:v>输入道路里程（km）</x:v>
+      </x:c>
       <x:c r="E22" s="10"/>
     </x:row>
-    <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="8" t="str">
+    <x:row r="23" ht="54" customHeight="1">
+      <x:c r="A23" s="21" t="str">
         <x:v>cway</x:v>
       </x:c>
-      <x:c r="B23" s="8" t="str">
+      <x:c r="B23" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C23" s="21" t="str">
         <x:v>Supplied carriageway</x:v>
       </x:c>
-      <x:c r="D23" s="8"/>
+      <x:c r="D23" s="21" t="str">
+        <x:v>输入车行道</x:v>
+      </x:c>
       <x:c r="E23" s="10"/>
     </x:row>
-    <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="8" t="str">
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" s="21" t="str">
         <x:v>start_slk</x:v>
       </x:c>
-      <x:c r="B24" s="8" t="str">
+      <x:c r="B24" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C24" s="21" t="str">
         <x:v>Official segment start SLK</x:v>
       </x:c>
-      <x:c r="D24" s="8"/>
+      <x:c r="D24" s="21" t="str">
+        <x:v>路段起点里程（km）</x:v>
+      </x:c>
       <x:c r="E24" s="10"/>
     </x:row>
-    <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="8" t="str">
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="21" t="str">
         <x:v>end_slk</x:v>
       </x:c>
-      <x:c r="B25" s="8" t="str">
+      <x:c r="B25" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C25" s="21" t="str">
         <x:v>Official segment end SLK</x:v>
       </x:c>
-      <x:c r="D25" s="8"/>
+      <x:c r="D25" s="21" t="str">
+        <x:v>路段终点里程（km）</x:v>
+      </x:c>
       <x:c r="E25" s="10"/>
     </x:row>
-    <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="8" t="str">
+    <x:row r="26" ht="54" customHeight="1">
+      <x:c r="A26" s="21" t="str">
         <x:v>latitude</x:v>
       </x:c>
-      <x:c r="B26" s="8" t="str">
+      <x:c r="B26" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C26" s="21" t="str">
         <x:v>Prediction point WGS84 latitude</x:v>
       </x:c>
-      <x:c r="D26" s="8"/>
+      <x:c r="D26" s="21" t="str">
+        <x:v>预测位置纬度</x:v>
+      </x:c>
       <x:c r="E26" s="10"/>
     </x:row>
-    <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="8" t="str">
+    <x:row r="27" ht="54" customHeight="1">
+      <x:c r="A27" s="21" t="str">
         <x:v>longitude</x:v>
       </x:c>
-      <x:c r="B27" s="8" t="str">
+      <x:c r="B27" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C27" s="21" t="str">
         <x:v>Prediction point WGS84 longitude</x:v>
       </x:c>
-      <x:c r="D27" s="8"/>
+      <x:c r="D27" s="21" t="str">
+        <x:v>预测位置经度</x:v>
+      </x:c>
       <x:c r="E27" s="10"/>
     </x:row>
-    <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="8" t="str">
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="A28" s="21" t="str">
         <x:v>matched_road_no</x:v>
       </x:c>
-      <x:c r="B28" s="8" t="str">
+      <x:c r="B28" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C28" s="21" t="str">
         <x:v>Road number resolved from measured geometry</x:v>
       </x:c>
-      <x:c r="D28" s="8"/>
+      <x:c r="D28" s="21" t="str">
+        <x:v>匹配道路编号</x:v>
+      </x:c>
       <x:c r="E28" s="10"/>
     </x:row>
-    <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="8" t="str">
+    <x:row r="29" ht="54" customHeight="1">
+      <x:c r="A29" s="21" t="str">
         <x:v>matched_slk_km</x:v>
       </x:c>
-      <x:c r="B29" s="8" t="str">
+      <x:c r="B29" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C29" s="21" t="str">
         <x:v>SLK resolved from measured geometry</x:v>
       </x:c>
-      <x:c r="D29" s="8"/>
+      <x:c r="D29" s="21" t="str">
+        <x:v>匹配道路里程（km）</x:v>
+      </x:c>
       <x:c r="E29" s="10"/>
     </x:row>
-    <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="8" t="str">
+    <x:row r="30" ht="54" customHeight="1">
+      <x:c r="A30" s="21" t="str">
         <x:v>matched_cway</x:v>
       </x:c>
-      <x:c r="B30" s="8" t="str">
+      <x:c r="B30" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C30" s="21" t="str">
         <x:v>Resolved carriageway</x:v>
       </x:c>
-      <x:c r="D30" s="8"/>
+      <x:c r="D30" s="21" t="str">
+        <x:v>匹配车行道</x:v>
+      </x:c>
       <x:c r="E30" s="10"/>
     </x:row>
-    <x:row r="31" ht="30" customHeight="1">
-      <x:c r="A31" s="8" t="str">
+    <x:row r="31" ht="54" customHeight="1">
+      <x:c r="A31" s="21" t="str">
         <x:v>road_offset_m</x:v>
       </x:c>
-      <x:c r="B31" s="8" t="str">
+      <x:c r="B31" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
       <x:c r="C31" s="21" t="str">
         <x:v>Distance from supplied coordinates to matched road in metres</x:v>
       </x:c>
-      <x:c r="D31" s="8"/>
+      <x:c r="D31" s="21" t="str">
+        <x:v>距匹配道路距离（m）</x:v>
+      </x:c>
       <x:c r="E31" s="10"/>
     </x:row>
-    <x:row r="32" ht="30" customHeight="1">
-      <x:c r="A32" s="8" t="str">
+    <x:row r="32" ht="54" customHeight="1">
+      <x:c r="A32" s="21" t="str">
         <x:v>location_status</x:v>
       </x:c>
-      <x:c r="B32" s="8" t="str">
+      <x:c r="B32" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="C32" s="21" t="str">
         <x:v>Road matching or input consistency outcome</x:v>
       </x:c>
-      <x:c r="D32" s="8"/>
+      <x:c r="D32" s="21" t="str">
+        <x:v>位置匹配状态</x:v>
+      </x:c>
       <x:c r="E32" s="10"/>
     </x:row>
-    <x:row r="33" ht="30" customHeight="1">
-      <x:c r="A33" s="8" t="str">
+    <x:row r="33" ht="54" customHeight="1">
+      <x:c r="A33" s="21" t="str">
+        <x:v>obs_peak_cross_ped_per_h</x:v>
+      </x:c>
+      <x:c r="B33" s="21" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C33" s="21" t="str">
+        <x:v>Observed peak-hour flow — Crossing. Optional input only; blank for unknown sites.</x:v>
+      </x:c>
+      <x:c r="D33" s="21" t="str">
+        <x:v>观测横穿高峰小时流量（可空）</x:v>
+      </x:c>
+      <x:c r="E33" s="10"/>
+    </x:row>
+    <x:row r="34" ht="54" customHeight="1">
+      <x:c r="A34" s="21" t="str">
         <x:v>pred_peak_cross_ped_per_h</x:v>
       </x:c>
-      <x:c r="B33" s="8" t="str">
+      <x:c r="B34" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
-      <x:c r="C33" s="21" t="str">
+      <x:c r="C34" s="21" t="str">
         <x:v>Predicted peak crossing pedestrians per hour</x:v>
       </x:c>
-      <x:c r="D33" s="8"/>
-      <x:c r="E33" s="10"/>
-    </x:row>
-    <x:row r="34" ht="30" customHeight="1">
-      <x:c r="A34" s="8" t="str">
+      <x:c r="D34" s="21" t="str">
+        <x:v>模型预测横穿高峰小时流量</x:v>
+      </x:c>
+      <x:c r="E34" s="10"/>
+    </x:row>
+    <x:row r="35" ht="54" customHeight="1">
+      <x:c r="A35" s="21" t="str">
+        <x:v>existing_irap_cross_recoded_ped_per_h</x:v>
+      </x:c>
+      <x:c r="B35" s="21" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C35" s="21" t="str">
+        <x:v>Existing iRAP flow estimate (recoded) — Crossing. Client recoding, then equal-weight source-row mean; not an official exact count.</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="str">
+        <x:v>现有 iRAP 横穿流量估计（换算值）</x:v>
+      </x:c>
+      <x:c r="E35" s="10"/>
+    </x:row>
+    <x:row r="36" ht="54" customHeight="1">
+      <x:c r="A36" s="21" t="str">
+        <x:v>observed_cross_category</x:v>
+      </x:c>
+      <x:c r="B36" s="21" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="C36" s="21" t="str">
+        <x:v>Observed flow category — Crossing. Project continuous upper-bound rule; raw count is unchanged.</x:v>
+      </x:c>
+      <x:c r="D36" s="21" t="str">
+        <x:v>观测横穿流量等级</x:v>
+      </x:c>
+      <x:c r="E36" s="10"/>
+    </x:row>
+    <x:row r="37" ht="54" customHeight="1">
+      <x:c r="A37" s="21" t="str">
+        <x:v>predicted_cross_category</x:v>
+      </x:c>
+      <x:c r="B37" s="21" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="C37" s="21" t="str">
+        <x:v>Model-predicted flow category — Crossing. Same continuous rule as observed categories.</x:v>
+      </x:c>
+      <x:c r="D37" s="21" t="str">
+        <x:v>模型预测横穿流量等级</x:v>
+      </x:c>
+      <x:c r="E37" s="10"/>
+    </x:row>
+    <x:row r="38" ht="54" customHeight="1">
+      <x:c r="A38" s="21" t="str">
+        <x:v>existing_ausrap_cross_category</x:v>
+      </x:c>
+      <x:c r="B38" s="21" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="C38" s="21" t="str">
+        <x:v>Existing AusRAP flow category — Crossing. Blank when categories are missing or mixed; details in comparison_notes.</x:v>
+      </x:c>
+      <x:c r="D38" s="21" t="str">
+        <x:v>现有 AusRAP 横穿流量等级</x:v>
+      </x:c>
+      <x:c r="E38" s="10"/>
+    </x:row>
+    <x:row r="39" ht="54" customHeight="1">
+      <x:c r="A39" s="21" t="str">
+        <x:v>existing_ausrap_cross_band</x:v>
+      </x:c>
+      <x:c r="B39" s="21" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C39" s="21" t="str">
+        <x:v>Existing AusRAP flow band — Crossing. Mean source endpoints when multiple records match; not a confidence interval.</x:v>
+      </x:c>
+      <x:c r="D39" s="21" t="str">
+        <x:v>现有 AusRAP 横穿流量区间</x:v>
+      </x:c>
+      <x:c r="E39" s="10"/>
+    </x:row>
+    <x:row r="40" ht="54" customHeight="1">
+      <x:c r="A40" s="21" t="str">
+        <x:v>obs_peak_along_ped_per_h</x:v>
+      </x:c>
+      <x:c r="B40" s="21" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C40" s="21" t="str">
+        <x:v>Observed peak-hour flow — Along-road. Optional input only; original survey coverage retained.</x:v>
+      </x:c>
+      <x:c r="D40" s="21" t="str">
+        <x:v>观测沿路高峰小时流量（可空）</x:v>
+      </x:c>
+      <x:c r="E40" s="10"/>
+    </x:row>
+    <x:row r="41" ht="54" customHeight="1">
+      <x:c r="A41" s="21" t="str">
         <x:v>pred_peak_along_ped_per_h</x:v>
       </x:c>
-      <x:c r="B34" s="8" t="str">
+      <x:c r="B41" s="21" t="str">
         <x:v>number</x:v>
       </x:c>
-      <x:c r="C34" s="21" t="str">
+      <x:c r="C41" s="21" t="str">
         <x:v>Predicted peak along-road pedestrians per hour</x:v>
       </x:c>
-      <x:c r="D34" s="8"/>
-      <x:c r="E34" s="10"/>
-    </x:row>
-    <x:row r="35" ht="30" customHeight="1">
-      <x:c r="A35" s="8" t="str">
+      <x:c r="D41" s="21" t="str">
+        <x:v>模型预测沿路高峰小时流量</x:v>
+      </x:c>
+      <x:c r="E41" s="10"/>
+    </x:row>
+    <x:row r="42" ht="54" customHeight="1">
+      <x:c r="A42" s="21" t="str">
+        <x:v>existing_irap_along_recoded_ped_per_h</x:v>
+      </x:c>
+      <x:c r="B42" s="21" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C42" s="21" t="str">
+        <x:v>Existing iRAP flow estimate (recoded) — Along-road. Sum both sides within each record, then average matched records.</x:v>
+      </x:c>
+      <x:c r="D42" s="21" t="str">
+        <x:v>现有 iRAP 沿路流量估计（换算值）</x:v>
+      </x:c>
+      <x:c r="E42" s="10"/>
+    </x:row>
+    <x:row r="43" ht="54" customHeight="1">
+      <x:c r="A43" s="21" t="str">
+        <x:v>existing_ausrap_along_combined_band</x:v>
+      </x:c>
+      <x:c r="B43" s="21" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C43" s="21" t="str">
+        <x:v>Existing AusRAP combined flow band — Along-road. Sum side endpoints, then average matched records.</x:v>
+      </x:c>
+      <x:c r="D43" s="21" t="str">
+        <x:v>现有 AusRAP 沿路合并流量区间</x:v>
+      </x:c>
+      <x:c r="E43" s="10"/>
+    </x:row>
+    <x:row r="44" ht="54" customHeight="1">
+      <x:c r="A44" s="21" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="B35" s="8" t="str">
+      <x:c r="B44" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
-      <x:c r="C35" s="21" t="str">
+      <x:c r="C44" s="21" t="str">
         <x:v>Prediction outcome</x:v>
       </x:c>
-      <x:c r="D35" s="8"/>
-      <x:c r="E35" s="10"/>
-    </x:row>
-    <x:row r="36" ht="30" customHeight="1">
-      <x:c r="A36" s="8" t="str">
+      <x:c r="D44" s="21" t="str">
+        <x:v>预测状态</x:v>
+      </x:c>
+      <x:c r="E44" s="10"/>
+    </x:row>
+    <x:row r="45" ht="54" customHeight="1">
+      <x:c r="A45" s="21" t="str">
         <x:v>message</x:v>
       </x:c>
-      <x:c r="B36" s="8" t="str">
+      <x:c r="B45" s="21" t="str">
         <x:v>text</x:v>
       </x:c>
-      <x:c r="C36" s="21" t="str">
+      <x:c r="C45" s="21" t="str">
         <x:v>Warning or failure details</x:v>
       </x:c>
-      <x:c r="D36" s="8"/>
-      <x:c r="E36" s="10"/>
-    </x:row>
-    <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="8"/>
-      <x:c r="B37" s="8"/>
-      <x:c r="C37" s="21"/>
-      <x:c r="D37" s="8"/>
-      <x:c r="E37" s="10"/>
-    </x:row>
-    <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="8"/>
-      <x:c r="B38" s="8"/>
-      <x:c r="C38" s="21"/>
-      <x:c r="D38" s="8"/>
-      <x:c r="E38" s="10"/>
-    </x:row>
-    <x:row r="39" ht="30" customHeight="1">
-      <x:c r="A39" s="8"/>
-      <x:c r="B39" s="8"/>
-      <x:c r="C39" s="21"/>
-      <x:c r="D39" s="8"/>
-      <x:c r="E39" s="10"/>
-    </x:row>
-    <x:row r="40" ht="30" customHeight="1">
-      <x:c r="A40" s="8"/>
-      <x:c r="B40" s="8"/>
-      <x:c r="C40" s="21"/>
-      <x:c r="D40" s="8"/>
-      <x:c r="E40" s="10"/>
-    </x:row>
-    <x:row r="41" ht="30" customHeight="1">
-      <x:c r="A41" s="8"/>
-      <x:c r="B41" s="8"/>
-      <x:c r="C41" s="21"/>
-      <x:c r="D41" s="8"/>
-      <x:c r="E41" s="10"/>
-    </x:row>
-    <x:row r="42" ht="30" customHeight="1">
-      <x:c r="A42" s="8"/>
-      <x:c r="B42" s="8"/>
-      <x:c r="C42" s="21"/>
-      <x:c r="D42" s="8"/>
-      <x:c r="E42" s="10"/>
-    </x:row>
-    <x:row r="43" ht="30" customHeight="1">
-      <x:c r="A43" s="8"/>
-      <x:c r="B43" s="8"/>
-      <x:c r="C43" s="21"/>
-      <x:c r="D43" s="8"/>
-      <x:c r="E43" s="10"/>
-    </x:row>
-    <x:row r="44" ht="30" customHeight="1">
-      <x:c r="A44" s="8"/>
-      <x:c r="B44" s="8"/>
-      <x:c r="C44" s="8"/>
-      <x:c r="D44" s="8"/>
-      <x:c r="E44" s="10"/>
-    </x:row>
-    <x:row r="45" ht="30" customHeight="1">
-      <x:c r="A45" s="8"/>
-      <x:c r="B45" s="8"/>
-      <x:c r="C45" s="8"/>
-      <x:c r="D45" s="8"/>
+      <x:c r="D45" s="21" t="str">
+        <x:v>预测说明</x:v>
+      </x:c>
       <x:c r="E45" s="10"/>
     </x:row>
-    <x:row r="46" ht="30" customHeight="1">
-      <x:c r="A46" s="8"/>
-      <x:c r="B46" s="8"/>
-      <x:c r="C46" s="8"/>
-      <x:c r="D46" s="8"/>
+    <x:row r="46" ht="54" customHeight="1">
+      <x:c r="A46" s="21" t="str">
+        <x:v>comparison_status</x:v>
+      </x:c>
+      <x:c r="B46" s="21" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C46" s="21" t="str">
+        <x:v>AusRAP reference matching/availability. Separate from model prediction status; does not measure accuracy.</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="str">
+        <x:v>AusRAP 对照状态</x:v>
+      </x:c>
       <x:c r="E46" s="10"/>
     </x:row>
-    <x:row r="47" ht="30" customHeight="1">
-      <x:c r="A47" s="8"/>
-      <x:c r="B47" s="8"/>
-      <x:c r="C47" s="8"/>
-      <x:c r="D47" s="8"/>
+    <x:row r="47" ht="54" customHeight="1">
+      <x:c r="A47" s="21" t="str">
+        <x:v>comparison_notes</x:v>
+      </x:c>
+      <x:c r="B47" s="21" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C47" s="21" t="str">
+        <x:v>AusRAP comparison notes: missing categories, multiple carriageways, mixed categories, source or matching problems.</x:v>
+      </x:c>
+      <x:c r="D47" s="21" t="str">
+        <x:v>AusRAP 对照说明</x:v>
+      </x:c>
       <x:c r="E47" s="10"/>
+    </x:row>
+    <x:row r="50" ht="40" customHeight="1">
+      <x:c r="A50" s="19" t="str">
+        <x:v>Reference source</x:v>
+      </x:c>
+      <x:c r="B50" s="19" t="str">
+        <x:v>data/raw/AusRAP Data - Words - MSDS.xlsx; source fingerprint and matched source rows are recorded in predictions.manifest.json.</x:v>
+      </x:c>
+      <x:c r="C50" s="19"/>
+      <x:c r="D50" s="19"/>
+    </x:row>
+    <x:row r="51" ht="40" customHeight="1">
+      <x:c r="A51" s="19" t="str">
+        <x:v>Matching rule</x:v>
+      </x:c>
+      <x:c r="B51" s="19" t="str">
+        <x:v>Point/segment-midpoint ±0.1 km, equal-weight mean, all source carriageways, inclusive direct-float overlap. Source record ID selects one row instead.</x:v>
+      </x:c>
+      <x:c r="C51" s="19"/>
+      <x:c r="D51" s="19"/>
+    </x:row>
+    <x:row r="52" ht="40" customHeight="1">
+      <x:c r="A52" s="19" t="str">
+        <x:v>Client recoding</x:v>
+      </x:c>
+      <x:c r="B52" s="19" t="str">
+        <x:v>1→0; 2→3; 3→15; 4→38; 5→75; 6→150; 7→250; 8→350; 9→450. No client recoding for 10/11.</x:v>
+      </x:c>
+      <x:c r="C52" s="19"/>
+      <x:c r="D52" s="19"/>
+    </x:row>
+    <x:row r="53" ht="40" customHeight="1">
+      <x:c r="A53" s="19" t="str">
+        <x:v>Category rule</x:v>
+      </x:c>
+      <x:c r="B53" s="19" t="str">
+        <x:v>positive_upper_bound_v1: zero separately; positive upper bounds 5,25,50,100,200,300,400,500,900. Project convention for continuous values.</x:v>
+      </x:c>
+      <x:c r="C53" s="19"/>
+      <x:c r="D53" s="19"/>
+    </x:row>
+    <x:row r="54" ht="40" customHeight="1">
+      <x:c r="A54" s="19" t="str">
+        <x:v>Reference manual</x:v>
+      </x:c>
+      <x:c r="B54" s="19" t="str">
+        <x:v>iRAP Star Rating and Investment Plan Manual v1.5 (2024), pp. 26,30–31; category endpoints only.</x:v>
+      </x:c>
+      <x:c r="C54" s="19"/>
+      <x:c r="D54" s="19"/>
+    </x:row>
+    <x:row r="55" ht="40" customHeight="1">
+      <x:c r="A55" s="19" t="str">
+        <x:v>Manual URL</x:v>
+      </x:c>
+      <x:c r="B55" s="19" t="str">
+        <x:v>https://austroads.gov.au/__data/assets/pdf_file/0033/836295/iRAP_Star_Rating_and_Investment_Plan_Manual_English.pdf</x:v>
+      </x:c>
+      <x:c r="C55" s="19"/>
+      <x:c r="D55" s="19"/>
+    </x:row>
+    <x:row r="56" ht="40" customHeight="1">
+      <x:c r="A56" s="19" t="str">
+        <x:v>Unknown sites</x:v>
+      </x:c>
+      <x:c r="B56" s="19" t="str">
+        <x:v>Observed counts/categories stay blank unless explicitly supplied. There are no MAE/RMSE or accuracy claims in this output.</x:v>
+      </x:c>
+      <x:c r="C56" s="19"/>
+      <x:c r="D56" s="19"/>
+    </x:row>
+    <x:row r="57" ht="40" customHeight="1">
+      <x:c r="A57" s="19" t="str">
+        <x:v>Units and absence</x:v>
+      </x:c>
+      <x:c r="B57" s="19" t="str">
+        <x:v>Counts and interval endpoints are pedestrians/hour. Blank means unavailable, not zero; 900+ represents an open upper bound.</x:v>
+      </x:c>
+      <x:c r="C57" s="19"/>
+      <x:c r="D57" s="19"/>
+    </x:row>
+    <x:row r="58" ht="40" customHeight="1">
+      <x:c r="A58" s="19" t="str">
+        <x:v>Optional source ID</x:v>
+      </x:c>
+      <x:c r="B58" s="19" t="str">
+        <x:v>ausrap_record_id = ausrap:&lt;source SHA-256&gt;:&lt;Excel row&gt;. This project identifier is tied to one source snapshot, not an official ID.</x:v>
+      </x:c>
+      <x:c r="C58" s="19"/>
+      <x:c r="D58" s="19"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -977,6 +1271,15 @@
     <x:mergeCell ref="B13:D13"/>
     <x:mergeCell ref="B14:D14"/>
     <x:mergeCell ref="A17:D17"/>
+    <x:mergeCell ref="B50:D50"/>
+    <x:mergeCell ref="B51:D51"/>
+    <x:mergeCell ref="B52:D52"/>
+    <x:mergeCell ref="B53:D53"/>
+    <x:mergeCell ref="B54:D54"/>
+    <x:mergeCell ref="B55:D55"/>
+    <x:mergeCell ref="B56:D56"/>
+    <x:mergeCell ref="B57:D57"/>
+    <x:mergeCell ref="B58:D58"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -997,15 +1300,26 @@
     <x:col min="11" max="14" width="14" style="13" customWidth="1"/>
     <x:col min="15" max="16" width="18" style="13" customWidth="1"/>
     <x:col min="17" max="19" width="22" style="13" customWidth="1"/>
-    <x:col min="20" max="20" width="15" style="13" customWidth="1"/>
+    <x:col min="20" max="20" width="25" style="13" hidden="0" customWidth="1"/>
     <x:col min="21" max="23" width="18" style="13" customWidth="1"/>
-    <x:col min="24" max="24" width="14" style="13" customWidth="1"/>
-    <x:col min="25" max="25" width="16" style="13" customWidth="1"/>
-    <x:col min="26" max="26" width="22" style="13" customWidth="1"/>
+    <x:col min="24" max="24" width="30" style="13" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="25" style="13" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="25" style="13" hidden="0" customWidth="1"/>
     <x:col min="27" max="16384" width="8.85155963897705" style="13" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="25" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="25" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="30" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="30" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="48" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="25" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="82" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="60" customHeight="1">
+    <x:row r="1" ht="74" customHeight="1">
       <x:c r="A1" s="22" t="str">
         <x:v>site_id</x:v>
       </x:c>
@@ -1048,26 +1362,51 @@
       <x:c r="N1" s="22" t="str">
         <x:v>location_status</x:v>
       </x:c>
-      <x:c r="O1" s="22" t="str">
+      <x:c r="O1" s="26" t="str">
+        <x:v>obs_peak_cross_ped_per_h</x:v>
+      </x:c>
+      <x:c r="P1" s="26" t="str">
         <x:v>pred_peak_cross_ped_per_h</x:v>
       </x:c>
-      <x:c r="P1" s="22" t="str">
+      <x:c r="Q1" s="26" t="str">
+        <x:v>existing_irap_cross_recoded_ped_per_h</x:v>
+      </x:c>
+      <x:c r="R1" s="26" t="str">
+        <x:v>observed_cross_category</x:v>
+      </x:c>
+      <x:c r="S1" s="36" t="str">
+        <x:v>predicted_cross_category</x:v>
+      </x:c>
+      <x:c r="T1" s="36" t="str">
+        <x:v>existing_ausrap_cross_category</x:v>
+      </x:c>
+      <x:c r="U1" s="36" t="str">
+        <x:v>existing_ausrap_cross_band</x:v>
+      </x:c>
+      <x:c r="V1" s="36" t="str">
+        <x:v>obs_peak_along_ped_per_h</x:v>
+      </x:c>
+      <x:c r="W1" s="36" t="str">
         <x:v>pred_peak_along_ped_per_h</x:v>
       </x:c>
-      <x:c r="Q1" s="22" t="str">
+      <x:c r="X1" s="36" t="str">
+        <x:v>existing_irap_along_recoded_ped_per_h</x:v>
+      </x:c>
+      <x:c r="Y1" s="36" t="str">
+        <x:v>existing_ausrap_along_combined_band</x:v>
+      </x:c>
+      <x:c r="Z1" s="36" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="R1" s="22" t="str">
+      <x:c r="AA1" s="36" t="str">
         <x:v>message</x:v>
       </x:c>
-      <x:c r="S1"/>
-      <x:c r="T1"/>
-      <x:c r="U1"/>
-      <x:c r="V1"/>
-      <x:c r="W1"/>
-      <x:c r="X1"/>
-      <x:c r="Y1"/>
-      <x:c r="Z1"/>
+      <x:c r="AB1" s="36" t="str">
+        <x:v>comparison_status</x:v>
+      </x:c>
+      <x:c r="AC1" s="36" t="str">
+        <x:v>comparison_notes</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="13.550000190734863" customHeight="1">
       <x:c r="A2" s="14"/>
@@ -1084,18 +1423,21 @@
       <x:c r="L2" s="16"/>
       <x:c r="M2" s="16"/>
       <x:c r="N2" s="16"/>
-      <x:c r="O2" s="17"/>
-      <x:c r="P2" s="17"/>
-      <x:c r="Q2" s="14"/>
-      <x:c r="R2" s="14"/>
-      <x:c r="S2"/>
-      <x:c r="T2"/>
-      <x:c r="U2"/>
-      <x:c r="V2"/>
-      <x:c r="W2"/>
-      <x:c r="X2"/>
-      <x:c r="Y2"/>
-      <x:c r="Z2"/>
+      <x:c r="O2" s="27"/>
+      <x:c r="P2" s="27"/>
+      <x:c r="Q2" s="27"/>
+      <x:c r="R2" s="39"/>
+      <x:c r="S2" s="40"/>
+      <x:c r="T2" s="40"/>
+      <x:c r="U2" s="37"/>
+      <x:c r="V2" s="38"/>
+      <x:c r="W2" s="38"/>
+      <x:c r="X2" s="38"/>
+      <x:c r="Y2" s="37"/>
+      <x:c r="Z2" s="37"/>
+      <x:c r="AA2" s="37"/>
+      <x:c r="AB2" s="37"/>
+      <x:c r="AC2" s="37"/>
     </x:row>
     <x:row r="3" ht="13.550000190734863" customHeight="1">
       <x:c r="A3" s="14"/>
@@ -1112,18 +1454,21 @@
       <x:c r="L3" s="16"/>
       <x:c r="M3" s="16"/>
       <x:c r="N3" s="16"/>
-      <x:c r="O3" s="17"/>
-      <x:c r="P3" s="17"/>
-      <x:c r="Q3" s="15"/>
-      <x:c r="R3" s="14"/>
-      <x:c r="S3"/>
-      <x:c r="T3"/>
-      <x:c r="U3"/>
-      <x:c r="V3"/>
-      <x:c r="W3"/>
-      <x:c r="X3"/>
-      <x:c r="Y3"/>
-      <x:c r="Z3"/>
+      <x:c r="O3" s="27"/>
+      <x:c r="P3" s="27"/>
+      <x:c r="Q3" s="27"/>
+      <x:c r="R3" s="39"/>
+      <x:c r="S3" s="40"/>
+      <x:c r="T3" s="40"/>
+      <x:c r="U3" s="37"/>
+      <x:c r="V3" s="38"/>
+      <x:c r="W3" s="38"/>
+      <x:c r="X3" s="38"/>
+      <x:c r="Y3" s="37"/>
+      <x:c r="Z3" s="37"/>
+      <x:c r="AA3" s="37"/>
+      <x:c r="AB3" s="37"/>
+      <x:c r="AC3" s="37"/>
     </x:row>
     <x:row r="4" ht="13.550000190734863" customHeight="1">
       <x:c r="A4" s="14"/>
@@ -1140,18 +1485,21 @@
       <x:c r="L4" s="16"/>
       <x:c r="M4" s="16"/>
       <x:c r="N4" s="16"/>
-      <x:c r="O4" s="17"/>
-      <x:c r="P4" s="17"/>
-      <x:c r="Q4" s="15"/>
-      <x:c r="R4" s="15"/>
-      <x:c r="S4"/>
-      <x:c r="T4"/>
-      <x:c r="U4"/>
-      <x:c r="V4"/>
-      <x:c r="W4"/>
-      <x:c r="X4"/>
-      <x:c r="Y4"/>
-      <x:c r="Z4"/>
+      <x:c r="O4" s="27"/>
+      <x:c r="P4" s="27"/>
+      <x:c r="Q4" s="27"/>
+      <x:c r="R4" s="39"/>
+      <x:c r="S4" s="40"/>
+      <x:c r="T4" s="40"/>
+      <x:c r="U4" s="37"/>
+      <x:c r="V4" s="38"/>
+      <x:c r="W4" s="38"/>
+      <x:c r="X4" s="38"/>
+      <x:c r="Y4" s="37"/>
+      <x:c r="Z4" s="37"/>
+      <x:c r="AA4" s="37"/>
+      <x:c r="AB4" s="37"/>
+      <x:c r="AC4" s="37"/>
     </x:row>
     <x:row r="5" ht="13.550000190734863" customHeight="1">
       <x:c r="A5" s="14"/>
@@ -1168,18 +1516,21 @@
       <x:c r="L5" s="16"/>
       <x:c r="M5" s="16"/>
       <x:c r="N5" s="16"/>
-      <x:c r="O5" s="17"/>
-      <x:c r="P5" s="17"/>
-      <x:c r="Q5" s="15"/>
-      <x:c r="R5" s="15"/>
-      <x:c r="S5"/>
-      <x:c r="T5"/>
-      <x:c r="U5"/>
-      <x:c r="V5"/>
-      <x:c r="W5"/>
-      <x:c r="X5"/>
-      <x:c r="Y5"/>
-      <x:c r="Z5"/>
+      <x:c r="O5" s="27"/>
+      <x:c r="P5" s="27"/>
+      <x:c r="Q5" s="27"/>
+      <x:c r="R5" s="39"/>
+      <x:c r="S5" s="40"/>
+      <x:c r="T5" s="40"/>
+      <x:c r="U5" s="37"/>
+      <x:c r="V5" s="38"/>
+      <x:c r="W5" s="38"/>
+      <x:c r="X5" s="38"/>
+      <x:c r="Y5" s="37"/>
+      <x:c r="Z5" s="37"/>
+      <x:c r="AA5" s="37"/>
+      <x:c r="AB5" s="37"/>
+      <x:c r="AC5" s="37"/>
     </x:row>
     <x:row r="6" ht="13.550000190734863" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -1196,18 +1547,21 @@
       <x:c r="L6" s="16"/>
       <x:c r="M6" s="16"/>
       <x:c r="N6" s="16"/>
-      <x:c r="O6" s="17"/>
-      <x:c r="P6" s="17"/>
-      <x:c r="Q6" s="15"/>
-      <x:c r="R6" s="15"/>
-      <x:c r="S6"/>
-      <x:c r="T6"/>
-      <x:c r="U6"/>
-      <x:c r="V6"/>
-      <x:c r="W6"/>
-      <x:c r="X6"/>
-      <x:c r="Y6"/>
-      <x:c r="Z6"/>
+      <x:c r="O6" s="27"/>
+      <x:c r="P6" s="27"/>
+      <x:c r="Q6" s="27"/>
+      <x:c r="R6" s="39"/>
+      <x:c r="S6" s="40"/>
+      <x:c r="T6" s="40"/>
+      <x:c r="U6" s="37"/>
+      <x:c r="V6" s="38"/>
+      <x:c r="W6" s="38"/>
+      <x:c r="X6" s="38"/>
+      <x:c r="Y6" s="37"/>
+      <x:c r="Z6" s="37"/>
+      <x:c r="AA6" s="37"/>
+      <x:c r="AB6" s="37"/>
+      <x:c r="AC6" s="37"/>
     </x:row>
     <x:row r="7" ht="13.550000190734863" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -1224,18 +1578,21 @@
       <x:c r="L7" s="16"/>
       <x:c r="M7" s="16"/>
       <x:c r="N7" s="16"/>
-      <x:c r="O7" s="17"/>
-      <x:c r="P7" s="17"/>
-      <x:c r="Q7" s="15"/>
-      <x:c r="R7" s="15"/>
-      <x:c r="S7"/>
-      <x:c r="T7"/>
-      <x:c r="U7"/>
-      <x:c r="V7"/>
-      <x:c r="W7"/>
-      <x:c r="X7"/>
-      <x:c r="Y7"/>
-      <x:c r="Z7"/>
+      <x:c r="O7" s="27"/>
+      <x:c r="P7" s="27"/>
+      <x:c r="Q7" s="27"/>
+      <x:c r="R7" s="39"/>
+      <x:c r="S7" s="40"/>
+      <x:c r="T7" s="40"/>
+      <x:c r="U7" s="37"/>
+      <x:c r="V7" s="38"/>
+      <x:c r="W7" s="38"/>
+      <x:c r="X7" s="38"/>
+      <x:c r="Y7" s="37"/>
+      <x:c r="Z7" s="37"/>
+      <x:c r="AA7" s="37"/>
+      <x:c r="AB7" s="37"/>
+      <x:c r="AC7" s="37"/>
     </x:row>
     <x:row r="8" ht="13.550000190734863" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -1252,18 +1609,21 @@
       <x:c r="L8" s="16"/>
       <x:c r="M8" s="16"/>
       <x:c r="N8" s="16"/>
-      <x:c r="O8" s="17"/>
-      <x:c r="P8" s="17"/>
-      <x:c r="Q8" s="15"/>
-      <x:c r="R8" s="14"/>
-      <x:c r="S8"/>
-      <x:c r="T8"/>
-      <x:c r="U8"/>
-      <x:c r="V8"/>
-      <x:c r="W8"/>
-      <x:c r="X8"/>
-      <x:c r="Y8"/>
-      <x:c r="Z8"/>
+      <x:c r="O8" s="27"/>
+      <x:c r="P8" s="27"/>
+      <x:c r="Q8" s="27"/>
+      <x:c r="R8" s="39"/>
+      <x:c r="S8" s="40"/>
+      <x:c r="T8" s="40"/>
+      <x:c r="U8" s="37"/>
+      <x:c r="V8" s="38"/>
+      <x:c r="W8" s="38"/>
+      <x:c r="X8" s="38"/>
+      <x:c r="Y8" s="37"/>
+      <x:c r="Z8" s="37"/>
+      <x:c r="AA8" s="37"/>
+      <x:c r="AB8" s="37"/>
+      <x:c r="AC8" s="37"/>
     </x:row>
     <x:row r="9" ht="13.550000190734863" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -1280,18 +1640,21 @@
       <x:c r="L9" s="16"/>
       <x:c r="M9" s="16"/>
       <x:c r="N9" s="16"/>
-      <x:c r="O9" s="17"/>
-      <x:c r="P9" s="17"/>
-      <x:c r="Q9" s="15"/>
-      <x:c r="R9" s="15"/>
-      <x:c r="S9"/>
-      <x:c r="T9"/>
-      <x:c r="U9"/>
-      <x:c r="V9"/>
-      <x:c r="W9"/>
-      <x:c r="X9"/>
-      <x:c r="Y9"/>
-      <x:c r="Z9"/>
+      <x:c r="O9" s="27"/>
+      <x:c r="P9" s="27"/>
+      <x:c r="Q9" s="27"/>
+      <x:c r="R9" s="39"/>
+      <x:c r="S9" s="40"/>
+      <x:c r="T9" s="40"/>
+      <x:c r="U9" s="37"/>
+      <x:c r="V9" s="38"/>
+      <x:c r="W9" s="38"/>
+      <x:c r="X9" s="38"/>
+      <x:c r="Y9" s="37"/>
+      <x:c r="Z9" s="37"/>
+      <x:c r="AA9" s="37"/>
+      <x:c r="AB9" s="37"/>
+      <x:c r="AC9" s="37"/>
     </x:row>
     <x:row r="10" ht="13.550000190734863" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -1308,18 +1671,21 @@
       <x:c r="L10" s="16"/>
       <x:c r="M10" s="16"/>
       <x:c r="N10" s="16"/>
-      <x:c r="O10" s="17"/>
-      <x:c r="P10" s="17"/>
-      <x:c r="Q10" s="15"/>
-      <x:c r="R10" s="15"/>
-      <x:c r="S10"/>
-      <x:c r="T10"/>
-      <x:c r="U10"/>
-      <x:c r="V10"/>
-      <x:c r="W10"/>
-      <x:c r="X10"/>
-      <x:c r="Y10"/>
-      <x:c r="Z10"/>
+      <x:c r="O10" s="27"/>
+      <x:c r="P10" s="27"/>
+      <x:c r="Q10" s="27"/>
+      <x:c r="R10" s="39"/>
+      <x:c r="S10" s="40"/>
+      <x:c r="T10" s="40"/>
+      <x:c r="U10" s="37"/>
+      <x:c r="V10" s="38"/>
+      <x:c r="W10" s="38"/>
+      <x:c r="X10" s="38"/>
+      <x:c r="Y10" s="37"/>
+      <x:c r="Z10" s="37"/>
+      <x:c r="AA10" s="37"/>
+      <x:c r="AB10" s="37"/>
+      <x:c r="AC10" s="37"/>
     </x:row>
     <x:row r="11" ht="13.550000190734863" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -1336,18 +1702,21 @@
       <x:c r="L11" s="16"/>
       <x:c r="M11" s="16"/>
       <x:c r="N11" s="16"/>
-      <x:c r="O11" s="17"/>
-      <x:c r="P11" s="17"/>
-      <x:c r="Q11" s="15"/>
-      <x:c r="R11" s="15"/>
-      <x:c r="S11"/>
-      <x:c r="T11"/>
-      <x:c r="U11"/>
-      <x:c r="V11"/>
-      <x:c r="W11"/>
-      <x:c r="X11"/>
-      <x:c r="Y11"/>
-      <x:c r="Z11"/>
+      <x:c r="O11" s="27"/>
+      <x:c r="P11" s="27"/>
+      <x:c r="Q11" s="27"/>
+      <x:c r="R11" s="39"/>
+      <x:c r="S11" s="40"/>
+      <x:c r="T11" s="40"/>
+      <x:c r="U11" s="37"/>
+      <x:c r="V11" s="38"/>
+      <x:c r="W11" s="38"/>
+      <x:c r="X11" s="38"/>
+      <x:c r="Y11" s="37"/>
+      <x:c r="Z11" s="37"/>
+      <x:c r="AA11" s="37"/>
+      <x:c r="AB11" s="37"/>
+      <x:c r="AC11" s="37"/>
     </x:row>
     <x:row r="12" ht="13.550000190734863" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -1364,18 +1733,21 @@
       <x:c r="L12" s="16"/>
       <x:c r="M12" s="16"/>
       <x:c r="N12" s="16"/>
-      <x:c r="O12" s="17"/>
-      <x:c r="P12" s="17"/>
-      <x:c r="Q12" s="15"/>
-      <x:c r="R12" s="15"/>
-      <x:c r="S12"/>
-      <x:c r="T12"/>
-      <x:c r="U12"/>
-      <x:c r="V12"/>
-      <x:c r="W12"/>
-      <x:c r="X12"/>
-      <x:c r="Y12"/>
-      <x:c r="Z12"/>
+      <x:c r="O12" s="27"/>
+      <x:c r="P12" s="27"/>
+      <x:c r="Q12" s="27"/>
+      <x:c r="R12" s="39"/>
+      <x:c r="S12" s="40"/>
+      <x:c r="T12" s="40"/>
+      <x:c r="U12" s="37"/>
+      <x:c r="V12" s="38"/>
+      <x:c r="W12" s="38"/>
+      <x:c r="X12" s="38"/>
+      <x:c r="Y12" s="37"/>
+      <x:c r="Z12" s="37"/>
+      <x:c r="AA12" s="37"/>
+      <x:c r="AB12" s="37"/>
+      <x:c r="AC12" s="37"/>
     </x:row>
     <x:row r="13" ht="13.550000190734863" customHeight="1">
       <x:c r="A13" s="14"/>
@@ -1392,18 +1764,21 @@
       <x:c r="L13" s="16"/>
       <x:c r="M13" s="16"/>
       <x:c r="N13" s="16"/>
-      <x:c r="O13" s="17"/>
-      <x:c r="P13" s="17"/>
-      <x:c r="Q13" s="15"/>
-      <x:c r="R13" s="15"/>
-      <x:c r="S13"/>
-      <x:c r="T13"/>
-      <x:c r="U13"/>
-      <x:c r="V13"/>
-      <x:c r="W13"/>
-      <x:c r="X13"/>
-      <x:c r="Y13"/>
-      <x:c r="Z13"/>
+      <x:c r="O13" s="27"/>
+      <x:c r="P13" s="27"/>
+      <x:c r="Q13" s="27"/>
+      <x:c r="R13" s="39"/>
+      <x:c r="S13" s="40"/>
+      <x:c r="T13" s="40"/>
+      <x:c r="U13" s="37"/>
+      <x:c r="V13" s="38"/>
+      <x:c r="W13" s="38"/>
+      <x:c r="X13" s="38"/>
+      <x:c r="Y13" s="37"/>
+      <x:c r="Z13" s="37"/>
+      <x:c r="AA13" s="37"/>
+      <x:c r="AB13" s="37"/>
+      <x:c r="AC13" s="37"/>
     </x:row>
     <x:row r="14" ht="13.550000190734863" customHeight="1">
       <x:c r="A14" s="14"/>
@@ -1420,18 +1795,21 @@
       <x:c r="L14" s="16"/>
       <x:c r="M14" s="16"/>
       <x:c r="N14" s="16"/>
-      <x:c r="O14" s="17"/>
-      <x:c r="P14" s="17"/>
-      <x:c r="Q14" s="15"/>
-      <x:c r="R14" s="15"/>
-      <x:c r="S14"/>
-      <x:c r="T14"/>
-      <x:c r="U14"/>
-      <x:c r="V14"/>
-      <x:c r="W14"/>
-      <x:c r="X14"/>
-      <x:c r="Y14"/>
-      <x:c r="Z14"/>
+      <x:c r="O14" s="27"/>
+      <x:c r="P14" s="27"/>
+      <x:c r="Q14" s="27"/>
+      <x:c r="R14" s="39"/>
+      <x:c r="S14" s="40"/>
+      <x:c r="T14" s="40"/>
+      <x:c r="U14" s="37"/>
+      <x:c r="V14" s="38"/>
+      <x:c r="W14" s="38"/>
+      <x:c r="X14" s="38"/>
+      <x:c r="Y14" s="37"/>
+      <x:c r="Z14" s="37"/>
+      <x:c r="AA14" s="37"/>
+      <x:c r="AB14" s="37"/>
+      <x:c r="AC14" s="37"/>
     </x:row>
     <x:row r="15" ht="13.550000190734863" customHeight="1">
       <x:c r="A15" s="14"/>
@@ -1448,18 +1826,21 @@
       <x:c r="L15" s="16"/>
       <x:c r="M15" s="16"/>
       <x:c r="N15" s="16"/>
-      <x:c r="O15" s="17"/>
-      <x:c r="P15" s="17"/>
-      <x:c r="Q15" s="15"/>
-      <x:c r="R15" s="15"/>
-      <x:c r="S15"/>
-      <x:c r="T15"/>
-      <x:c r="U15"/>
-      <x:c r="V15"/>
-      <x:c r="W15"/>
-      <x:c r="X15"/>
-      <x:c r="Y15"/>
-      <x:c r="Z15"/>
+      <x:c r="O15" s="27"/>
+      <x:c r="P15" s="27"/>
+      <x:c r="Q15" s="27"/>
+      <x:c r="R15" s="39"/>
+      <x:c r="S15" s="40"/>
+      <x:c r="T15" s="40"/>
+      <x:c r="U15" s="37"/>
+      <x:c r="V15" s="38"/>
+      <x:c r="W15" s="38"/>
+      <x:c r="X15" s="38"/>
+      <x:c r="Y15" s="37"/>
+      <x:c r="Z15" s="37"/>
+      <x:c r="AA15" s="37"/>
+      <x:c r="AB15" s="37"/>
+      <x:c r="AC15" s="37"/>
     </x:row>
     <x:row r="16" ht="13.550000190734863" customHeight="1">
       <x:c r="A16" s="14"/>
@@ -1476,18 +1857,21 @@
       <x:c r="L16" s="16"/>
       <x:c r="M16" s="16"/>
       <x:c r="N16" s="16"/>
-      <x:c r="O16" s="17"/>
-      <x:c r="P16" s="17"/>
-      <x:c r="Q16" s="14"/>
-      <x:c r="R16" s="14"/>
-      <x:c r="S16"/>
-      <x:c r="T16"/>
-      <x:c r="U16"/>
-      <x:c r="V16"/>
-      <x:c r="W16"/>
-      <x:c r="X16"/>
-      <x:c r="Y16"/>
-      <x:c r="Z16"/>
+      <x:c r="O16" s="27"/>
+      <x:c r="P16" s="27"/>
+      <x:c r="Q16" s="27"/>
+      <x:c r="R16" s="39"/>
+      <x:c r="S16" s="40"/>
+      <x:c r="T16" s="40"/>
+      <x:c r="U16" s="37"/>
+      <x:c r="V16" s="38"/>
+      <x:c r="W16" s="38"/>
+      <x:c r="X16" s="38"/>
+      <x:c r="Y16" s="37"/>
+      <x:c r="Z16" s="37"/>
+      <x:c r="AA16" s="37"/>
+      <x:c r="AB16" s="37"/>
+      <x:c r="AC16" s="37"/>
     </x:row>
     <x:row r="17" ht="13.550000190734863" customHeight="1">
       <x:c r="A17" s="14"/>
@@ -1504,18 +1888,21 @@
       <x:c r="L17" s="16"/>
       <x:c r="M17" s="16"/>
       <x:c r="N17" s="16"/>
-      <x:c r="O17" s="17"/>
-      <x:c r="P17" s="17"/>
-      <x:c r="Q17" s="15"/>
-      <x:c r="R17" s="15"/>
-      <x:c r="S17"/>
-      <x:c r="T17"/>
-      <x:c r="U17"/>
-      <x:c r="V17"/>
-      <x:c r="W17"/>
-      <x:c r="X17"/>
-      <x:c r="Y17"/>
-      <x:c r="Z17"/>
+      <x:c r="O17" s="27"/>
+      <x:c r="P17" s="27"/>
+      <x:c r="Q17" s="27"/>
+      <x:c r="R17" s="39"/>
+      <x:c r="S17" s="40"/>
+      <x:c r="T17" s="40"/>
+      <x:c r="U17" s="37"/>
+      <x:c r="V17" s="38"/>
+      <x:c r="W17" s="38"/>
+      <x:c r="X17" s="38"/>
+      <x:c r="Y17" s="37"/>
+      <x:c r="Z17" s="37"/>
+      <x:c r="AA17" s="37"/>
+      <x:c r="AB17" s="37"/>
+      <x:c r="AC17" s="37"/>
     </x:row>
     <x:row r="18" ht="13.550000190734863" customHeight="1">
       <x:c r="A18" s="14"/>
@@ -1532,18 +1919,21 @@
       <x:c r="L18" s="16"/>
       <x:c r="M18" s="16"/>
       <x:c r="N18" s="16"/>
-      <x:c r="O18" s="17"/>
-      <x:c r="P18" s="17"/>
-      <x:c r="Q18" s="14"/>
-      <x:c r="R18" s="14"/>
-      <x:c r="S18"/>
-      <x:c r="T18"/>
-      <x:c r="U18"/>
-      <x:c r="V18"/>
-      <x:c r="W18"/>
-      <x:c r="X18"/>
-      <x:c r="Y18"/>
-      <x:c r="Z18"/>
+      <x:c r="O18" s="27"/>
+      <x:c r="P18" s="27"/>
+      <x:c r="Q18" s="27"/>
+      <x:c r="R18" s="39"/>
+      <x:c r="S18" s="40"/>
+      <x:c r="T18" s="40"/>
+      <x:c r="U18" s="37"/>
+      <x:c r="V18" s="38"/>
+      <x:c r="W18" s="38"/>
+      <x:c r="X18" s="38"/>
+      <x:c r="Y18" s="37"/>
+      <x:c r="Z18" s="37"/>
+      <x:c r="AA18" s="37"/>
+      <x:c r="AB18" s="37"/>
+      <x:c r="AC18" s="37"/>
     </x:row>
     <x:row r="19" ht="13.550000190734863" customHeight="1">
       <x:c r="A19" s="14"/>
@@ -1560,18 +1950,21 @@
       <x:c r="L19" s="16"/>
       <x:c r="M19" s="16"/>
       <x:c r="N19" s="16"/>
-      <x:c r="O19" s="17"/>
-      <x:c r="P19" s="17"/>
-      <x:c r="Q19" s="15"/>
-      <x:c r="R19" s="15"/>
-      <x:c r="S19"/>
-      <x:c r="T19"/>
-      <x:c r="U19"/>
-      <x:c r="V19"/>
-      <x:c r="W19"/>
-      <x:c r="X19"/>
-      <x:c r="Y19"/>
-      <x:c r="Z19"/>
+      <x:c r="O19" s="27"/>
+      <x:c r="P19" s="27"/>
+      <x:c r="Q19" s="27"/>
+      <x:c r="R19" s="39"/>
+      <x:c r="S19" s="40"/>
+      <x:c r="T19" s="40"/>
+      <x:c r="U19" s="37"/>
+      <x:c r="V19" s="38"/>
+      <x:c r="W19" s="38"/>
+      <x:c r="X19" s="38"/>
+      <x:c r="Y19" s="37"/>
+      <x:c r="Z19" s="37"/>
+      <x:c r="AA19" s="37"/>
+      <x:c r="AB19" s="37"/>
+      <x:c r="AC19" s="37"/>
     </x:row>
     <x:row r="20" ht="13.550000190734863" customHeight="1">
       <x:c r="A20" s="14"/>
@@ -1588,18 +1981,21 @@
       <x:c r="L20" s="16"/>
       <x:c r="M20" s="16"/>
       <x:c r="N20" s="16"/>
-      <x:c r="O20" s="17"/>
-      <x:c r="P20" s="17"/>
-      <x:c r="Q20" s="14"/>
-      <x:c r="R20" s="14"/>
-      <x:c r="S20"/>
-      <x:c r="T20"/>
-      <x:c r="U20"/>
-      <x:c r="V20"/>
-      <x:c r="W20"/>
-      <x:c r="X20"/>
-      <x:c r="Y20"/>
-      <x:c r="Z20"/>
+      <x:c r="O20" s="27"/>
+      <x:c r="P20" s="27"/>
+      <x:c r="Q20" s="27"/>
+      <x:c r="R20" s="39"/>
+      <x:c r="S20" s="40"/>
+      <x:c r="T20" s="40"/>
+      <x:c r="U20" s="37"/>
+      <x:c r="V20" s="38"/>
+      <x:c r="W20" s="38"/>
+      <x:c r="X20" s="38"/>
+      <x:c r="Y20" s="37"/>
+      <x:c r="Z20" s="37"/>
+      <x:c r="AA20" s="37"/>
+      <x:c r="AB20" s="37"/>
+      <x:c r="AC20" s="37"/>
     </x:row>
     <x:row r="21" ht="13.550000190734863" customHeight="1">
       <x:c r="A21" s="14"/>
@@ -1616,18 +2012,21 @@
       <x:c r="L21" s="16"/>
       <x:c r="M21" s="16"/>
       <x:c r="N21" s="16"/>
-      <x:c r="O21" s="17"/>
-      <x:c r="P21" s="17"/>
-      <x:c r="Q21" s="15"/>
-      <x:c r="R21" s="14"/>
-      <x:c r="S21"/>
-      <x:c r="T21"/>
-      <x:c r="U21"/>
-      <x:c r="V21"/>
-      <x:c r="W21"/>
-      <x:c r="X21"/>
-      <x:c r="Y21"/>
-      <x:c r="Z21"/>
+      <x:c r="O21" s="27"/>
+      <x:c r="P21" s="27"/>
+      <x:c r="Q21" s="27"/>
+      <x:c r="R21" s="39"/>
+      <x:c r="S21" s="40"/>
+      <x:c r="T21" s="40"/>
+      <x:c r="U21" s="37"/>
+      <x:c r="V21" s="38"/>
+      <x:c r="W21" s="38"/>
+      <x:c r="X21" s="38"/>
+      <x:c r="Y21" s="37"/>
+      <x:c r="Z21" s="37"/>
+      <x:c r="AA21" s="37"/>
+      <x:c r="AB21" s="37"/>
+      <x:c r="AC21" s="37"/>
     </x:row>
     <x:row r="22" ht="13.550000190734863" customHeight="1">
       <x:c r="A22" s="14"/>
@@ -1644,18 +2043,21 @@
       <x:c r="L22" s="16"/>
       <x:c r="M22" s="16"/>
       <x:c r="N22" s="16"/>
-      <x:c r="O22" s="17"/>
-      <x:c r="P22" s="17"/>
-      <x:c r="Q22" s="15"/>
-      <x:c r="R22" s="15"/>
-      <x:c r="S22"/>
-      <x:c r="T22"/>
-      <x:c r="U22"/>
-      <x:c r="V22"/>
-      <x:c r="W22"/>
-      <x:c r="X22"/>
-      <x:c r="Y22"/>
-      <x:c r="Z22"/>
+      <x:c r="O22" s="27"/>
+      <x:c r="P22" s="27"/>
+      <x:c r="Q22" s="27"/>
+      <x:c r="R22" s="39"/>
+      <x:c r="S22" s="40"/>
+      <x:c r="T22" s="40"/>
+      <x:c r="U22" s="37"/>
+      <x:c r="V22" s="38"/>
+      <x:c r="W22" s="38"/>
+      <x:c r="X22" s="38"/>
+      <x:c r="Y22" s="37"/>
+      <x:c r="Z22" s="37"/>
+      <x:c r="AA22" s="37"/>
+      <x:c r="AB22" s="37"/>
+      <x:c r="AC22" s="37"/>
     </x:row>
     <x:row r="23" ht="13.550000190734863" customHeight="1">
       <x:c r="A23" s="14"/>
@@ -1672,18 +2074,21 @@
       <x:c r="L23" s="16"/>
       <x:c r="M23" s="16"/>
       <x:c r="N23" s="16"/>
-      <x:c r="O23" s="17"/>
-      <x:c r="P23" s="17"/>
-      <x:c r="Q23" s="15"/>
-      <x:c r="R23" s="14"/>
-      <x:c r="S23"/>
-      <x:c r="T23"/>
-      <x:c r="U23"/>
-      <x:c r="V23"/>
-      <x:c r="W23"/>
-      <x:c r="X23"/>
-      <x:c r="Y23"/>
-      <x:c r="Z23"/>
+      <x:c r="O23" s="27"/>
+      <x:c r="P23" s="27"/>
+      <x:c r="Q23" s="27"/>
+      <x:c r="R23" s="39"/>
+      <x:c r="S23" s="40"/>
+      <x:c r="T23" s="40"/>
+      <x:c r="U23" s="37"/>
+      <x:c r="V23" s="38"/>
+      <x:c r="W23" s="38"/>
+      <x:c r="X23" s="38"/>
+      <x:c r="Y23" s="37"/>
+      <x:c r="Z23" s="37"/>
+      <x:c r="AA23" s="37"/>
+      <x:c r="AB23" s="37"/>
+      <x:c r="AC23" s="37"/>
     </x:row>
     <x:row r="24" ht="13.550000190734863" customHeight="1">
       <x:c r="A24" s="14"/>
@@ -1700,18 +2105,21 @@
       <x:c r="L24" s="16"/>
       <x:c r="M24" s="16"/>
       <x:c r="N24" s="16"/>
-      <x:c r="O24" s="17"/>
-      <x:c r="P24" s="17"/>
-      <x:c r="Q24" s="15"/>
-      <x:c r="R24" s="14"/>
-      <x:c r="S24"/>
-      <x:c r="T24"/>
-      <x:c r="U24"/>
-      <x:c r="V24"/>
-      <x:c r="W24"/>
-      <x:c r="X24"/>
-      <x:c r="Y24"/>
-      <x:c r="Z24"/>
+      <x:c r="O24" s="27"/>
+      <x:c r="P24" s="27"/>
+      <x:c r="Q24" s="27"/>
+      <x:c r="R24" s="39"/>
+      <x:c r="S24" s="40"/>
+      <x:c r="T24" s="40"/>
+      <x:c r="U24" s="37"/>
+      <x:c r="V24" s="38"/>
+      <x:c r="W24" s="38"/>
+      <x:c r="X24" s="38"/>
+      <x:c r="Y24" s="37"/>
+      <x:c r="Z24" s="37"/>
+      <x:c r="AA24" s="37"/>
+      <x:c r="AB24" s="37"/>
+      <x:c r="AC24" s="37"/>
     </x:row>
     <x:row r="25" ht="13.550000190734863" customHeight="1">
       <x:c r="A25" s="14"/>
@@ -1728,18 +2136,21 @@
       <x:c r="L25" s="16"/>
       <x:c r="M25" s="16"/>
       <x:c r="N25" s="16"/>
-      <x:c r="O25" s="17"/>
-      <x:c r="P25" s="17"/>
-      <x:c r="Q25" s="15"/>
-      <x:c r="R25" s="14"/>
-      <x:c r="S25"/>
-      <x:c r="T25"/>
-      <x:c r="U25"/>
-      <x:c r="V25"/>
-      <x:c r="W25"/>
-      <x:c r="X25"/>
-      <x:c r="Y25"/>
-      <x:c r="Z25"/>
+      <x:c r="O25" s="27"/>
+      <x:c r="P25" s="27"/>
+      <x:c r="Q25" s="27"/>
+      <x:c r="R25" s="39"/>
+      <x:c r="S25" s="40"/>
+      <x:c r="T25" s="40"/>
+      <x:c r="U25" s="37"/>
+      <x:c r="V25" s="38"/>
+      <x:c r="W25" s="38"/>
+      <x:c r="X25" s="38"/>
+      <x:c r="Y25" s="37"/>
+      <x:c r="Z25" s="37"/>
+      <x:c r="AA25" s="37"/>
+      <x:c r="AB25" s="37"/>
+      <x:c r="AC25" s="37"/>
     </x:row>
     <x:row r="26" ht="13.550000190734863" customHeight="1">
       <x:c r="A26" s="14"/>
@@ -1756,18 +2167,21 @@
       <x:c r="L26" s="16"/>
       <x:c r="M26" s="16"/>
       <x:c r="N26" s="16"/>
-      <x:c r="O26" s="17"/>
-      <x:c r="P26" s="17"/>
-      <x:c r="Q26" s="15"/>
-      <x:c r="R26" s="15"/>
-      <x:c r="S26"/>
-      <x:c r="T26"/>
-      <x:c r="U26"/>
-      <x:c r="V26"/>
-      <x:c r="W26"/>
-      <x:c r="X26"/>
-      <x:c r="Y26"/>
-      <x:c r="Z26"/>
+      <x:c r="O26" s="27"/>
+      <x:c r="P26" s="27"/>
+      <x:c r="Q26" s="27"/>
+      <x:c r="R26" s="39"/>
+      <x:c r="S26" s="40"/>
+      <x:c r="T26" s="40"/>
+      <x:c r="U26" s="37"/>
+      <x:c r="V26" s="38"/>
+      <x:c r="W26" s="38"/>
+      <x:c r="X26" s="38"/>
+      <x:c r="Y26" s="37"/>
+      <x:c r="Z26" s="37"/>
+      <x:c r="AA26" s="37"/>
+      <x:c r="AB26" s="37"/>
+      <x:c r="AC26" s="37"/>
     </x:row>
     <x:row r="27" ht="13.550000190734863" customHeight="1">
       <x:c r="A27" s="14"/>
@@ -1784,18 +2198,21 @@
       <x:c r="L27" s="16"/>
       <x:c r="M27" s="16"/>
       <x:c r="N27" s="16"/>
-      <x:c r="O27" s="17"/>
-      <x:c r="P27" s="17"/>
-      <x:c r="Q27" s="15"/>
-      <x:c r="R27" s="14"/>
-      <x:c r="S27"/>
-      <x:c r="T27"/>
-      <x:c r="U27"/>
-      <x:c r="V27"/>
-      <x:c r="W27"/>
-      <x:c r="X27"/>
-      <x:c r="Y27"/>
-      <x:c r="Z27"/>
+      <x:c r="O27" s="27"/>
+      <x:c r="P27" s="27"/>
+      <x:c r="Q27" s="27"/>
+      <x:c r="R27" s="39"/>
+      <x:c r="S27" s="40"/>
+      <x:c r="T27" s="40"/>
+      <x:c r="U27" s="37"/>
+      <x:c r="V27" s="38"/>
+      <x:c r="W27" s="38"/>
+      <x:c r="X27" s="38"/>
+      <x:c r="Y27" s="37"/>
+      <x:c r="Z27" s="37"/>
+      <x:c r="AA27" s="37"/>
+      <x:c r="AB27" s="37"/>
+      <x:c r="AC27" s="37"/>
     </x:row>
     <x:row r="28" ht="13.550000190734863" customHeight="1">
       <x:c r="A28" s="14"/>
@@ -1812,18 +2229,21 @@
       <x:c r="L28" s="16"/>
       <x:c r="M28" s="16"/>
       <x:c r="N28" s="16"/>
-      <x:c r="O28" s="17"/>
-      <x:c r="P28" s="17"/>
-      <x:c r="Q28" s="15"/>
-      <x:c r="R28" s="15"/>
-      <x:c r="S28"/>
-      <x:c r="T28"/>
-      <x:c r="U28"/>
-      <x:c r="V28"/>
-      <x:c r="W28"/>
-      <x:c r="X28"/>
-      <x:c r="Y28"/>
-      <x:c r="Z28"/>
+      <x:c r="O28" s="27"/>
+      <x:c r="P28" s="27"/>
+      <x:c r="Q28" s="27"/>
+      <x:c r="R28" s="39"/>
+      <x:c r="S28" s="40"/>
+      <x:c r="T28" s="40"/>
+      <x:c r="U28" s="37"/>
+      <x:c r="V28" s="38"/>
+      <x:c r="W28" s="38"/>
+      <x:c r="X28" s="38"/>
+      <x:c r="Y28" s="37"/>
+      <x:c r="Z28" s="37"/>
+      <x:c r="AA28" s="37"/>
+      <x:c r="AB28" s="37"/>
+      <x:c r="AC28" s="37"/>
     </x:row>
     <x:row r="29" ht="13.550000190734863" customHeight="1">
       <x:c r="A29" s="14"/>
@@ -1840,18 +2260,21 @@
       <x:c r="L29" s="16"/>
       <x:c r="M29" s="16"/>
       <x:c r="N29" s="16"/>
-      <x:c r="O29" s="17"/>
-      <x:c r="P29" s="17"/>
-      <x:c r="Q29" s="15"/>
-      <x:c r="R29" s="15"/>
-      <x:c r="S29"/>
-      <x:c r="T29"/>
-      <x:c r="U29"/>
-      <x:c r="V29"/>
-      <x:c r="W29"/>
-      <x:c r="X29"/>
-      <x:c r="Y29"/>
-      <x:c r="Z29"/>
+      <x:c r="O29" s="27"/>
+      <x:c r="P29" s="27"/>
+      <x:c r="Q29" s="27"/>
+      <x:c r="R29" s="39"/>
+      <x:c r="S29" s="40"/>
+      <x:c r="T29" s="40"/>
+      <x:c r="U29" s="37"/>
+      <x:c r="V29" s="38"/>
+      <x:c r="W29" s="38"/>
+      <x:c r="X29" s="38"/>
+      <x:c r="Y29" s="37"/>
+      <x:c r="Z29" s="37"/>
+      <x:c r="AA29" s="37"/>
+      <x:c r="AB29" s="37"/>
+      <x:c r="AC29" s="37"/>
     </x:row>
     <x:row r="30" ht="13.550000190734863" customHeight="1">
       <x:c r="A30" s="14"/>
@@ -1868,18 +2291,21 @@
       <x:c r="L30" s="16"/>
       <x:c r="M30" s="16"/>
       <x:c r="N30" s="16"/>
-      <x:c r="O30" s="17"/>
-      <x:c r="P30" s="17"/>
-      <x:c r="Q30" s="15"/>
-      <x:c r="R30" s="15"/>
-      <x:c r="S30"/>
-      <x:c r="T30"/>
-      <x:c r="U30"/>
-      <x:c r="V30"/>
-      <x:c r="W30"/>
-      <x:c r="X30"/>
-      <x:c r="Y30"/>
-      <x:c r="Z30"/>
+      <x:c r="O30" s="27"/>
+      <x:c r="P30" s="27"/>
+      <x:c r="Q30" s="27"/>
+      <x:c r="R30" s="39"/>
+      <x:c r="S30" s="40"/>
+      <x:c r="T30" s="40"/>
+      <x:c r="U30" s="37"/>
+      <x:c r="V30" s="38"/>
+      <x:c r="W30" s="38"/>
+      <x:c r="X30" s="38"/>
+      <x:c r="Y30" s="37"/>
+      <x:c r="Z30" s="37"/>
+      <x:c r="AA30" s="37"/>
+      <x:c r="AB30" s="37"/>
+      <x:c r="AC30" s="37"/>
     </x:row>
     <x:row r="31" ht="13.550000190734863" customHeight="1">
       <x:c r="A31" s="14"/>
@@ -1896,18 +2322,21 @@
       <x:c r="L31" s="16"/>
       <x:c r="M31" s="16"/>
       <x:c r="N31" s="16"/>
-      <x:c r="O31" s="17"/>
-      <x:c r="P31" s="17"/>
-      <x:c r="Q31" s="15"/>
-      <x:c r="R31" s="14"/>
-      <x:c r="S31"/>
-      <x:c r="T31"/>
-      <x:c r="U31"/>
-      <x:c r="V31"/>
-      <x:c r="W31"/>
-      <x:c r="X31"/>
-      <x:c r="Y31"/>
-      <x:c r="Z31"/>
+      <x:c r="O31" s="27"/>
+      <x:c r="P31" s="27"/>
+      <x:c r="Q31" s="27"/>
+      <x:c r="R31" s="39"/>
+      <x:c r="S31" s="40"/>
+      <x:c r="T31" s="40"/>
+      <x:c r="U31" s="37"/>
+      <x:c r="V31" s="38"/>
+      <x:c r="W31" s="38"/>
+      <x:c r="X31" s="38"/>
+      <x:c r="Y31" s="37"/>
+      <x:c r="Z31" s="37"/>
+      <x:c r="AA31" s="37"/>
+      <x:c r="AB31" s="37"/>
+      <x:c r="AC31" s="37"/>
     </x:row>
     <x:row r="32" ht="13.550000190734863" customHeight="1">
       <x:c r="A32" s="14"/>
@@ -1924,18 +2353,21 @@
       <x:c r="L32" s="16"/>
       <x:c r="M32" s="16"/>
       <x:c r="N32" s="16"/>
-      <x:c r="O32" s="17"/>
-      <x:c r="P32" s="17"/>
-      <x:c r="Q32" s="15"/>
-      <x:c r="R32" s="15"/>
-      <x:c r="S32"/>
-      <x:c r="T32"/>
-      <x:c r="U32"/>
-      <x:c r="V32"/>
-      <x:c r="W32"/>
-      <x:c r="X32"/>
-      <x:c r="Y32"/>
-      <x:c r="Z32"/>
+      <x:c r="O32" s="27"/>
+      <x:c r="P32" s="27"/>
+      <x:c r="Q32" s="27"/>
+      <x:c r="R32" s="39"/>
+      <x:c r="S32" s="40"/>
+      <x:c r="T32" s="40"/>
+      <x:c r="U32" s="37"/>
+      <x:c r="V32" s="38"/>
+      <x:c r="W32" s="38"/>
+      <x:c r="X32" s="38"/>
+      <x:c r="Y32" s="37"/>
+      <x:c r="Z32" s="37"/>
+      <x:c r="AA32" s="37"/>
+      <x:c r="AB32" s="37"/>
+      <x:c r="AC32" s="37"/>
     </x:row>
     <x:row r="33" ht="13.550000190734863" customHeight="1">
       <x:c r="A33" s="14"/>
@@ -1952,18 +2384,21 @@
       <x:c r="L33" s="16"/>
       <x:c r="M33" s="16"/>
       <x:c r="N33" s="16"/>
-      <x:c r="O33" s="17"/>
-      <x:c r="P33" s="17"/>
-      <x:c r="Q33" s="15"/>
-      <x:c r="R33" s="15"/>
-      <x:c r="S33"/>
-      <x:c r="T33"/>
-      <x:c r="U33"/>
-      <x:c r="V33"/>
-      <x:c r="W33"/>
-      <x:c r="X33"/>
-      <x:c r="Y33"/>
-      <x:c r="Z33"/>
+      <x:c r="O33" s="27"/>
+      <x:c r="P33" s="27"/>
+      <x:c r="Q33" s="27"/>
+      <x:c r="R33" s="39"/>
+      <x:c r="S33" s="40"/>
+      <x:c r="T33" s="40"/>
+      <x:c r="U33" s="37"/>
+      <x:c r="V33" s="38"/>
+      <x:c r="W33" s="38"/>
+      <x:c r="X33" s="38"/>
+      <x:c r="Y33" s="37"/>
+      <x:c r="Z33" s="37"/>
+      <x:c r="AA33" s="37"/>
+      <x:c r="AB33" s="37"/>
+      <x:c r="AC33" s="37"/>
     </x:row>
     <x:row r="34" ht="13.550000190734863" customHeight="1">
       <x:c r="A34" s="14"/>
@@ -1980,18 +2415,21 @@
       <x:c r="L34" s="16"/>
       <x:c r="M34" s="16"/>
       <x:c r="N34" s="16"/>
-      <x:c r="O34" s="17"/>
-      <x:c r="P34" s="17"/>
-      <x:c r="Q34" s="15"/>
-      <x:c r="R34" s="15"/>
-      <x:c r="S34"/>
-      <x:c r="T34"/>
-      <x:c r="U34"/>
-      <x:c r="V34"/>
-      <x:c r="W34"/>
-      <x:c r="X34"/>
-      <x:c r="Y34"/>
-      <x:c r="Z34"/>
+      <x:c r="O34" s="27"/>
+      <x:c r="P34" s="27"/>
+      <x:c r="Q34" s="27"/>
+      <x:c r="R34" s="39"/>
+      <x:c r="S34" s="40"/>
+      <x:c r="T34" s="40"/>
+      <x:c r="U34" s="37"/>
+      <x:c r="V34" s="38"/>
+      <x:c r="W34" s="38"/>
+      <x:c r="X34" s="38"/>
+      <x:c r="Y34" s="37"/>
+      <x:c r="Z34" s="37"/>
+      <x:c r="AA34" s="37"/>
+      <x:c r="AB34" s="37"/>
+      <x:c r="AC34" s="37"/>
     </x:row>
     <x:row r="35" ht="13.550000190734863" customHeight="1">
       <x:c r="A35" s="14"/>
@@ -2008,18 +2446,21 @@
       <x:c r="L35" s="16"/>
       <x:c r="M35" s="16"/>
       <x:c r="N35" s="16"/>
-      <x:c r="O35" s="17"/>
-      <x:c r="P35" s="17"/>
-      <x:c r="Q35" s="15"/>
-      <x:c r="R35" s="15"/>
-      <x:c r="S35"/>
-      <x:c r="T35"/>
-      <x:c r="U35"/>
-      <x:c r="V35"/>
-      <x:c r="W35"/>
-      <x:c r="X35"/>
-      <x:c r="Y35"/>
-      <x:c r="Z35"/>
+      <x:c r="O35" s="27"/>
+      <x:c r="P35" s="27"/>
+      <x:c r="Q35" s="27"/>
+      <x:c r="R35" s="39"/>
+      <x:c r="S35" s="40"/>
+      <x:c r="T35" s="40"/>
+      <x:c r="U35" s="37"/>
+      <x:c r="V35" s="38"/>
+      <x:c r="W35" s="38"/>
+      <x:c r="X35" s="38"/>
+      <x:c r="Y35" s="37"/>
+      <x:c r="Z35" s="37"/>
+      <x:c r="AA35" s="37"/>
+      <x:c r="AB35" s="37"/>
+      <x:c r="AC35" s="37"/>
     </x:row>
     <x:row r="36" ht="13.550000190734863" customHeight="1">
       <x:c r="A36" s="14"/>
@@ -2036,18 +2477,21 @@
       <x:c r="L36" s="16"/>
       <x:c r="M36" s="16"/>
       <x:c r="N36" s="16"/>
-      <x:c r="O36" s="17"/>
-      <x:c r="P36" s="17"/>
-      <x:c r="Q36" s="15"/>
-      <x:c r="R36" s="14"/>
-      <x:c r="S36"/>
-      <x:c r="T36"/>
-      <x:c r="U36"/>
-      <x:c r="V36"/>
-      <x:c r="W36"/>
-      <x:c r="X36"/>
-      <x:c r="Y36"/>
-      <x:c r="Z36"/>
+      <x:c r="O36" s="27"/>
+      <x:c r="P36" s="27"/>
+      <x:c r="Q36" s="27"/>
+      <x:c r="R36" s="39"/>
+      <x:c r="S36" s="40"/>
+      <x:c r="T36" s="40"/>
+      <x:c r="U36" s="37"/>
+      <x:c r="V36" s="38"/>
+      <x:c r="W36" s="38"/>
+      <x:c r="X36" s="38"/>
+      <x:c r="Y36" s="37"/>
+      <x:c r="Z36" s="37"/>
+      <x:c r="AA36" s="37"/>
+      <x:c r="AB36" s="37"/>
+      <x:c r="AC36" s="37"/>
     </x:row>
     <x:row r="37" ht="13.550000190734863" customHeight="1">
       <x:c r="A37" s="14"/>
@@ -2064,18 +2508,21 @@
       <x:c r="L37" s="16"/>
       <x:c r="M37" s="16"/>
       <x:c r="N37" s="16"/>
-      <x:c r="O37" s="17"/>
-      <x:c r="P37" s="17"/>
-      <x:c r="Q37" s="15"/>
-      <x:c r="R37" s="14"/>
-      <x:c r="S37"/>
-      <x:c r="T37"/>
-      <x:c r="U37"/>
-      <x:c r="V37"/>
-      <x:c r="W37"/>
-      <x:c r="X37"/>
-      <x:c r="Y37"/>
-      <x:c r="Z37"/>
+      <x:c r="O37" s="27"/>
+      <x:c r="P37" s="27"/>
+      <x:c r="Q37" s="27"/>
+      <x:c r="R37" s="39"/>
+      <x:c r="S37" s="40"/>
+      <x:c r="T37" s="40"/>
+      <x:c r="U37" s="37"/>
+      <x:c r="V37" s="38"/>
+      <x:c r="W37" s="38"/>
+      <x:c r="X37" s="38"/>
+      <x:c r="Y37" s="37"/>
+      <x:c r="Z37" s="37"/>
+      <x:c r="AA37" s="37"/>
+      <x:c r="AB37" s="37"/>
+      <x:c r="AC37" s="37"/>
     </x:row>
     <x:row r="38" ht="13.550000190734863" customHeight="1">
       <x:c r="A38" s="14"/>
@@ -2092,18 +2539,21 @@
       <x:c r="L38" s="16"/>
       <x:c r="M38" s="16"/>
       <x:c r="N38" s="16"/>
-      <x:c r="O38" s="17"/>
-      <x:c r="P38" s="17"/>
-      <x:c r="Q38" s="15"/>
-      <x:c r="R38" s="15"/>
-      <x:c r="S38"/>
-      <x:c r="T38"/>
-      <x:c r="U38"/>
-      <x:c r="V38"/>
-      <x:c r="W38"/>
-      <x:c r="X38"/>
-      <x:c r="Y38"/>
-      <x:c r="Z38"/>
+      <x:c r="O38" s="27"/>
+      <x:c r="P38" s="27"/>
+      <x:c r="Q38" s="27"/>
+      <x:c r="R38" s="39"/>
+      <x:c r="S38" s="40"/>
+      <x:c r="T38" s="40"/>
+      <x:c r="U38" s="37"/>
+      <x:c r="V38" s="38"/>
+      <x:c r="W38" s="38"/>
+      <x:c r="X38" s="38"/>
+      <x:c r="Y38" s="37"/>
+      <x:c r="Z38" s="37"/>
+      <x:c r="AA38" s="37"/>
+      <x:c r="AB38" s="37"/>
+      <x:c r="AC38" s="37"/>
     </x:row>
     <x:row r="39" ht="13.550000190734863" customHeight="1">
       <x:c r="A39" s="14"/>
@@ -2120,18 +2570,21 @@
       <x:c r="L39" s="16"/>
       <x:c r="M39" s="16"/>
       <x:c r="N39" s="16"/>
-      <x:c r="O39" s="17"/>
-      <x:c r="P39" s="17"/>
-      <x:c r="Q39" s="15"/>
-      <x:c r="R39" s="15"/>
-      <x:c r="S39"/>
-      <x:c r="T39"/>
-      <x:c r="U39"/>
-      <x:c r="V39"/>
-      <x:c r="W39"/>
-      <x:c r="X39"/>
-      <x:c r="Y39"/>
-      <x:c r="Z39"/>
+      <x:c r="O39" s="27"/>
+      <x:c r="P39" s="27"/>
+      <x:c r="Q39" s="27"/>
+      <x:c r="R39" s="39"/>
+      <x:c r="S39" s="40"/>
+      <x:c r="T39" s="40"/>
+      <x:c r="U39" s="37"/>
+      <x:c r="V39" s="38"/>
+      <x:c r="W39" s="38"/>
+      <x:c r="X39" s="38"/>
+      <x:c r="Y39" s="37"/>
+      <x:c r="Z39" s="37"/>
+      <x:c r="AA39" s="37"/>
+      <x:c r="AB39" s="37"/>
+      <x:c r="AC39" s="37"/>
     </x:row>
     <x:row r="40" ht="13.550000190734863" customHeight="1">
       <x:c r="A40" s="14"/>
@@ -2148,18 +2601,21 @@
       <x:c r="L40" s="16"/>
       <x:c r="M40" s="16"/>
       <x:c r="N40" s="16"/>
-      <x:c r="O40" s="17"/>
-      <x:c r="P40" s="17"/>
-      <x:c r="Q40" s="15"/>
-      <x:c r="R40" s="15"/>
-      <x:c r="S40"/>
-      <x:c r="T40"/>
-      <x:c r="U40"/>
-      <x:c r="V40"/>
-      <x:c r="W40"/>
-      <x:c r="X40"/>
-      <x:c r="Y40"/>
-      <x:c r="Z40"/>
+      <x:c r="O40" s="27"/>
+      <x:c r="P40" s="27"/>
+      <x:c r="Q40" s="27"/>
+      <x:c r="R40" s="39"/>
+      <x:c r="S40" s="40"/>
+      <x:c r="T40" s="40"/>
+      <x:c r="U40" s="37"/>
+      <x:c r="V40" s="38"/>
+      <x:c r="W40" s="38"/>
+      <x:c r="X40" s="38"/>
+      <x:c r="Y40" s="37"/>
+      <x:c r="Z40" s="37"/>
+      <x:c r="AA40" s="37"/>
+      <x:c r="AB40" s="37"/>
+      <x:c r="AC40" s="37"/>
     </x:row>
     <x:row r="41" ht="13.550000190734863" customHeight="1">
       <x:c r="A41" s="14"/>
@@ -2176,18 +2632,21 @@
       <x:c r="L41" s="16"/>
       <x:c r="M41" s="16"/>
       <x:c r="N41" s="16"/>
-      <x:c r="O41" s="17"/>
-      <x:c r="P41" s="17"/>
-      <x:c r="Q41" s="15"/>
-      <x:c r="R41" s="15"/>
-      <x:c r="S41"/>
-      <x:c r="T41"/>
-      <x:c r="U41"/>
-      <x:c r="V41"/>
-      <x:c r="W41"/>
-      <x:c r="X41"/>
-      <x:c r="Y41"/>
-      <x:c r="Z41"/>
+      <x:c r="O41" s="27"/>
+      <x:c r="P41" s="27"/>
+      <x:c r="Q41" s="27"/>
+      <x:c r="R41" s="39"/>
+      <x:c r="S41" s="40"/>
+      <x:c r="T41" s="40"/>
+      <x:c r="U41" s="37"/>
+      <x:c r="V41" s="38"/>
+      <x:c r="W41" s="38"/>
+      <x:c r="X41" s="38"/>
+      <x:c r="Y41" s="37"/>
+      <x:c r="Z41" s="37"/>
+      <x:c r="AA41" s="37"/>
+      <x:c r="AB41" s="37"/>
+      <x:c r="AC41" s="37"/>
     </x:row>
     <x:row r="42" ht="13.550000190734863" customHeight="1">
       <x:c r="A42" s="14"/>
@@ -2204,18 +2663,21 @@
       <x:c r="L42" s="16"/>
       <x:c r="M42" s="16"/>
       <x:c r="N42" s="16"/>
-      <x:c r="O42" s="17"/>
-      <x:c r="P42" s="17"/>
-      <x:c r="Q42" s="15"/>
-      <x:c r="R42" s="15"/>
-      <x:c r="S42"/>
-      <x:c r="T42"/>
-      <x:c r="U42"/>
-      <x:c r="V42"/>
-      <x:c r="W42"/>
-      <x:c r="X42"/>
-      <x:c r="Y42"/>
-      <x:c r="Z42"/>
+      <x:c r="O42" s="27"/>
+      <x:c r="P42" s="27"/>
+      <x:c r="Q42" s="27"/>
+      <x:c r="R42" s="39"/>
+      <x:c r="S42" s="40"/>
+      <x:c r="T42" s="40"/>
+      <x:c r="U42" s="37"/>
+      <x:c r="V42" s="38"/>
+      <x:c r="W42" s="38"/>
+      <x:c r="X42" s="38"/>
+      <x:c r="Y42" s="37"/>
+      <x:c r="Z42" s="37"/>
+      <x:c r="AA42" s="37"/>
+      <x:c r="AB42" s="37"/>
+      <x:c r="AC42" s="37"/>
     </x:row>
     <x:row r="43" ht="13.550000190734863" customHeight="1">
       <x:c r="A43" s="14"/>
@@ -2232,18 +2694,21 @@
       <x:c r="L43" s="16"/>
       <x:c r="M43" s="16"/>
       <x:c r="N43" s="16"/>
-      <x:c r="O43" s="17"/>
-      <x:c r="P43" s="17"/>
-      <x:c r="Q43" s="15"/>
-      <x:c r="R43" s="15"/>
-      <x:c r="S43"/>
-      <x:c r="T43"/>
-      <x:c r="U43"/>
-      <x:c r="V43"/>
-      <x:c r="W43"/>
-      <x:c r="X43"/>
-      <x:c r="Y43"/>
-      <x:c r="Z43"/>
+      <x:c r="O43" s="27"/>
+      <x:c r="P43" s="27"/>
+      <x:c r="Q43" s="27"/>
+      <x:c r="R43" s="39"/>
+      <x:c r="S43" s="40"/>
+      <x:c r="T43" s="40"/>
+      <x:c r="U43" s="37"/>
+      <x:c r="V43" s="38"/>
+      <x:c r="W43" s="38"/>
+      <x:c r="X43" s="38"/>
+      <x:c r="Y43" s="37"/>
+      <x:c r="Z43" s="37"/>
+      <x:c r="AA43" s="37"/>
+      <x:c r="AB43" s="37"/>
+      <x:c r="AC43" s="37"/>
     </x:row>
     <x:row r="44" ht="13.550000190734863" customHeight="1">
       <x:c r="A44" s="14"/>
@@ -2260,18 +2725,21 @@
       <x:c r="L44" s="16"/>
       <x:c r="M44" s="16"/>
       <x:c r="N44" s="16"/>
-      <x:c r="O44" s="17"/>
-      <x:c r="P44" s="17"/>
-      <x:c r="Q44" s="15"/>
-      <x:c r="R44" s="15"/>
-      <x:c r="S44"/>
-      <x:c r="T44"/>
-      <x:c r="U44"/>
-      <x:c r="V44"/>
-      <x:c r="W44"/>
-      <x:c r="X44"/>
-      <x:c r="Y44"/>
-      <x:c r="Z44"/>
+      <x:c r="O44" s="27"/>
+      <x:c r="P44" s="27"/>
+      <x:c r="Q44" s="27"/>
+      <x:c r="R44" s="39"/>
+      <x:c r="S44" s="40"/>
+      <x:c r="T44" s="40"/>
+      <x:c r="U44" s="37"/>
+      <x:c r="V44" s="38"/>
+      <x:c r="W44" s="38"/>
+      <x:c r="X44" s="38"/>
+      <x:c r="Y44" s="37"/>
+      <x:c r="Z44" s="37"/>
+      <x:c r="AA44" s="37"/>
+      <x:c r="AB44" s="37"/>
+      <x:c r="AC44" s="37"/>
     </x:row>
     <x:row r="45" ht="13.550000190734863" customHeight="1">
       <x:c r="A45" s="14"/>
@@ -2288,18 +2756,21 @@
       <x:c r="L45" s="16"/>
       <x:c r="M45" s="16"/>
       <x:c r="N45" s="16"/>
-      <x:c r="O45" s="17"/>
-      <x:c r="P45" s="17"/>
-      <x:c r="Q45" s="15"/>
-      <x:c r="R45" s="15"/>
-      <x:c r="S45"/>
-      <x:c r="T45"/>
-      <x:c r="U45"/>
-      <x:c r="V45"/>
-      <x:c r="W45"/>
-      <x:c r="X45"/>
-      <x:c r="Y45"/>
-      <x:c r="Z45"/>
+      <x:c r="O45" s="27"/>
+      <x:c r="P45" s="27"/>
+      <x:c r="Q45" s="27"/>
+      <x:c r="R45" s="39"/>
+      <x:c r="S45" s="40"/>
+      <x:c r="T45" s="40"/>
+      <x:c r="U45" s="37"/>
+      <x:c r="V45" s="38"/>
+      <x:c r="W45" s="38"/>
+      <x:c r="X45" s="38"/>
+      <x:c r="Y45" s="37"/>
+      <x:c r="Z45" s="37"/>
+      <x:c r="AA45" s="37"/>
+      <x:c r="AB45" s="37"/>
+      <x:c r="AC45" s="37"/>
     </x:row>
     <x:row r="46" ht="13.550000190734863" customHeight="1">
       <x:c r="A46" s="14"/>
@@ -2316,18 +2787,21 @@
       <x:c r="L46" s="16"/>
       <x:c r="M46" s="16"/>
       <x:c r="N46" s="16"/>
-      <x:c r="O46" s="17"/>
-      <x:c r="P46" s="17"/>
-      <x:c r="Q46" s="15"/>
-      <x:c r="R46" s="15"/>
-      <x:c r="S46"/>
-      <x:c r="T46"/>
-      <x:c r="U46"/>
-      <x:c r="V46"/>
-      <x:c r="W46"/>
-      <x:c r="X46"/>
-      <x:c r="Y46"/>
-      <x:c r="Z46"/>
+      <x:c r="O46" s="27"/>
+      <x:c r="P46" s="27"/>
+      <x:c r="Q46" s="27"/>
+      <x:c r="R46" s="39"/>
+      <x:c r="S46" s="40"/>
+      <x:c r="T46" s="40"/>
+      <x:c r="U46" s="37"/>
+      <x:c r="V46" s="38"/>
+      <x:c r="W46" s="38"/>
+      <x:c r="X46" s="38"/>
+      <x:c r="Y46" s="37"/>
+      <x:c r="Z46" s="37"/>
+      <x:c r="AA46" s="37"/>
+      <x:c r="AB46" s="37"/>
+      <x:c r="AC46" s="37"/>
     </x:row>
     <x:row r="47" ht="13.550000190734863" customHeight="1">
       <x:c r="A47" s="14"/>
@@ -2344,18 +2818,21 @@
       <x:c r="L47" s="16"/>
       <x:c r="M47" s="16"/>
       <x:c r="N47" s="16"/>
-      <x:c r="O47" s="17"/>
-      <x:c r="P47" s="17"/>
-      <x:c r="Q47" s="15"/>
-      <x:c r="R47" s="15"/>
-      <x:c r="S47"/>
-      <x:c r="T47"/>
-      <x:c r="U47"/>
-      <x:c r="V47"/>
-      <x:c r="W47"/>
-      <x:c r="X47"/>
-      <x:c r="Y47"/>
-      <x:c r="Z47"/>
+      <x:c r="O47" s="27"/>
+      <x:c r="P47" s="27"/>
+      <x:c r="Q47" s="27"/>
+      <x:c r="R47" s="39"/>
+      <x:c r="S47" s="40"/>
+      <x:c r="T47" s="40"/>
+      <x:c r="U47" s="37"/>
+      <x:c r="V47" s="38"/>
+      <x:c r="W47" s="38"/>
+      <x:c r="X47" s="38"/>
+      <x:c r="Y47" s="37"/>
+      <x:c r="Z47" s="37"/>
+      <x:c r="AA47" s="37"/>
+      <x:c r="AB47" s="37"/>
+      <x:c r="AC47" s="37"/>
     </x:row>
     <x:row r="48" ht="13.550000190734863" customHeight="1">
       <x:c r="A48" s="14"/>
@@ -2372,18 +2849,21 @@
       <x:c r="L48" s="16"/>
       <x:c r="M48" s="16"/>
       <x:c r="N48" s="16"/>
-      <x:c r="O48" s="17"/>
-      <x:c r="P48" s="17"/>
-      <x:c r="Q48" s="15"/>
-      <x:c r="R48" s="15"/>
-      <x:c r="S48"/>
-      <x:c r="T48"/>
-      <x:c r="U48"/>
-      <x:c r="V48"/>
-      <x:c r="W48"/>
-      <x:c r="X48"/>
-      <x:c r="Y48"/>
-      <x:c r="Z48"/>
+      <x:c r="O48" s="27"/>
+      <x:c r="P48" s="27"/>
+      <x:c r="Q48" s="27"/>
+      <x:c r="R48" s="39"/>
+      <x:c r="S48" s="40"/>
+      <x:c r="T48" s="40"/>
+      <x:c r="U48" s="37"/>
+      <x:c r="V48" s="38"/>
+      <x:c r="W48" s="38"/>
+      <x:c r="X48" s="38"/>
+      <x:c r="Y48" s="37"/>
+      <x:c r="Z48" s="37"/>
+      <x:c r="AA48" s="37"/>
+      <x:c r="AB48" s="37"/>
+      <x:c r="AC48" s="37"/>
     </x:row>
     <x:row r="49" ht="13.550000190734863" customHeight="1">
       <x:c r="A49" s="14"/>
@@ -2400,18 +2880,21 @@
       <x:c r="L49" s="16"/>
       <x:c r="M49" s="16"/>
       <x:c r="N49" s="16"/>
-      <x:c r="O49" s="17"/>
-      <x:c r="P49" s="17"/>
-      <x:c r="Q49" s="15"/>
-      <x:c r="R49" s="15"/>
-      <x:c r="S49"/>
-      <x:c r="T49"/>
-      <x:c r="U49"/>
-      <x:c r="V49"/>
-      <x:c r="W49"/>
-      <x:c r="X49"/>
-      <x:c r="Y49"/>
-      <x:c r="Z49"/>
+      <x:c r="O49" s="27"/>
+      <x:c r="P49" s="27"/>
+      <x:c r="Q49" s="27"/>
+      <x:c r="R49" s="39"/>
+      <x:c r="S49" s="40"/>
+      <x:c r="T49" s="40"/>
+      <x:c r="U49" s="37"/>
+      <x:c r="V49" s="38"/>
+      <x:c r="W49" s="38"/>
+      <x:c r="X49" s="38"/>
+      <x:c r="Y49" s="37"/>
+      <x:c r="Z49" s="37"/>
+      <x:c r="AA49" s="37"/>
+      <x:c r="AB49" s="37"/>
+      <x:c r="AC49" s="37"/>
     </x:row>
     <x:row r="50" ht="13.550000190734863" customHeight="1">
       <x:c r="A50" s="14"/>
@@ -2428,18 +2911,21 @@
       <x:c r="L50" s="16"/>
       <x:c r="M50" s="16"/>
       <x:c r="N50" s="16"/>
-      <x:c r="O50" s="17"/>
-      <x:c r="P50" s="17"/>
-      <x:c r="Q50" s="15"/>
-      <x:c r="R50" s="14"/>
-      <x:c r="S50"/>
-      <x:c r="T50"/>
-      <x:c r="U50"/>
-      <x:c r="V50"/>
-      <x:c r="W50"/>
-      <x:c r="X50"/>
-      <x:c r="Y50"/>
-      <x:c r="Z50"/>
+      <x:c r="O50" s="27"/>
+      <x:c r="P50" s="27"/>
+      <x:c r="Q50" s="27"/>
+      <x:c r="R50" s="39"/>
+      <x:c r="S50" s="40"/>
+      <x:c r="T50" s="40"/>
+      <x:c r="U50" s="37"/>
+      <x:c r="V50" s="38"/>
+      <x:c r="W50" s="38"/>
+      <x:c r="X50" s="38"/>
+      <x:c r="Y50" s="37"/>
+      <x:c r="Z50" s="37"/>
+      <x:c r="AA50" s="37"/>
+      <x:c r="AB50" s="37"/>
+      <x:c r="AC50" s="37"/>
     </x:row>
     <x:row r="51" ht="13.550000190734863" customHeight="1">
       <x:c r="A51" s="14"/>
@@ -2456,18 +2942,21 @@
       <x:c r="L51" s="16"/>
       <x:c r="M51" s="16"/>
       <x:c r="N51" s="16"/>
-      <x:c r="O51" s="17"/>
-      <x:c r="P51" s="17"/>
-      <x:c r="Q51" s="15"/>
-      <x:c r="R51" s="15"/>
-      <x:c r="S51"/>
-      <x:c r="T51"/>
-      <x:c r="U51"/>
-      <x:c r="V51"/>
-      <x:c r="W51"/>
-      <x:c r="X51"/>
-      <x:c r="Y51"/>
-      <x:c r="Z51"/>
+      <x:c r="O51" s="27"/>
+      <x:c r="P51" s="27"/>
+      <x:c r="Q51" s="27"/>
+      <x:c r="R51" s="39"/>
+      <x:c r="S51" s="40"/>
+      <x:c r="T51" s="40"/>
+      <x:c r="U51" s="37"/>
+      <x:c r="V51" s="38"/>
+      <x:c r="W51" s="38"/>
+      <x:c r="X51" s="38"/>
+      <x:c r="Y51" s="37"/>
+      <x:c r="Z51" s="37"/>
+      <x:c r="AA51" s="37"/>
+      <x:c r="AB51" s="37"/>
+      <x:c r="AC51" s="37"/>
     </x:row>
     <x:row r="52" ht="13.550000190734863" customHeight="1">
       <x:c r="A52" s="14"/>
@@ -2484,18 +2973,21 @@
       <x:c r="L52" s="16"/>
       <x:c r="M52" s="16"/>
       <x:c r="N52" s="16"/>
-      <x:c r="O52" s="17"/>
-      <x:c r="P52" s="17"/>
-      <x:c r="Q52" s="15"/>
-      <x:c r="R52" s="14"/>
-      <x:c r="S52"/>
-      <x:c r="T52"/>
-      <x:c r="U52"/>
-      <x:c r="V52"/>
-      <x:c r="W52"/>
-      <x:c r="X52"/>
-      <x:c r="Y52"/>
-      <x:c r="Z52"/>
+      <x:c r="O52" s="27"/>
+      <x:c r="P52" s="27"/>
+      <x:c r="Q52" s="27"/>
+      <x:c r="R52" s="39"/>
+      <x:c r="S52" s="40"/>
+      <x:c r="T52" s="40"/>
+      <x:c r="U52" s="37"/>
+      <x:c r="V52" s="38"/>
+      <x:c r="W52" s="38"/>
+      <x:c r="X52" s="38"/>
+      <x:c r="Y52" s="37"/>
+      <x:c r="Z52" s="37"/>
+      <x:c r="AA52" s="37"/>
+      <x:c r="AB52" s="37"/>
+      <x:c r="AC52" s="37"/>
     </x:row>
     <x:row r="53" ht="13.550000190734863" customHeight="1">
       <x:c r="A53" s="14"/>
@@ -2512,18 +3004,21 @@
       <x:c r="L53" s="16"/>
       <x:c r="M53" s="16"/>
       <x:c r="N53" s="16"/>
-      <x:c r="O53" s="17"/>
-      <x:c r="P53" s="17"/>
-      <x:c r="Q53" s="15"/>
-      <x:c r="R53" s="14"/>
-      <x:c r="S53"/>
-      <x:c r="T53"/>
-      <x:c r="U53"/>
-      <x:c r="V53"/>
-      <x:c r="W53"/>
-      <x:c r="X53"/>
-      <x:c r="Y53"/>
-      <x:c r="Z53"/>
+      <x:c r="O53" s="27"/>
+      <x:c r="P53" s="27"/>
+      <x:c r="Q53" s="27"/>
+      <x:c r="R53" s="39"/>
+      <x:c r="S53" s="40"/>
+      <x:c r="T53" s="40"/>
+      <x:c r="U53" s="37"/>
+      <x:c r="V53" s="38"/>
+      <x:c r="W53" s="38"/>
+      <x:c r="X53" s="38"/>
+      <x:c r="Y53" s="37"/>
+      <x:c r="Z53" s="37"/>
+      <x:c r="AA53" s="37"/>
+      <x:c r="AB53" s="37"/>
+      <x:c r="AC53" s="37"/>
     </x:row>
     <x:row r="54" ht="13.550000190734863" customHeight="1">
       <x:c r="A54" s="14"/>
@@ -2540,18 +3035,21 @@
       <x:c r="L54" s="16"/>
       <x:c r="M54" s="16"/>
       <x:c r="N54" s="16"/>
-      <x:c r="O54" s="17"/>
-      <x:c r="P54" s="17"/>
-      <x:c r="Q54" s="14"/>
-      <x:c r="R54" s="14"/>
-      <x:c r="S54"/>
-      <x:c r="T54"/>
-      <x:c r="U54"/>
-      <x:c r="V54"/>
-      <x:c r="W54"/>
-      <x:c r="X54"/>
-      <x:c r="Y54"/>
-      <x:c r="Z54"/>
+      <x:c r="O54" s="27"/>
+      <x:c r="P54" s="27"/>
+      <x:c r="Q54" s="27"/>
+      <x:c r="R54" s="39"/>
+      <x:c r="S54" s="40"/>
+      <x:c r="T54" s="40"/>
+      <x:c r="U54" s="37"/>
+      <x:c r="V54" s="38"/>
+      <x:c r="W54" s="38"/>
+      <x:c r="X54" s="38"/>
+      <x:c r="Y54" s="37"/>
+      <x:c r="Z54" s="37"/>
+      <x:c r="AA54" s="37"/>
+      <x:c r="AB54" s="37"/>
+      <x:c r="AC54" s="37"/>
     </x:row>
     <x:row r="55" ht="13.550000190734863" customHeight="1">
       <x:c r="A55" s="14"/>
@@ -2568,18 +3066,21 @@
       <x:c r="L55" s="16"/>
       <x:c r="M55" s="16"/>
       <x:c r="N55" s="16"/>
-      <x:c r="O55" s="17"/>
-      <x:c r="P55" s="17"/>
-      <x:c r="Q55" s="14"/>
-      <x:c r="R55" s="14"/>
-      <x:c r="S55"/>
-      <x:c r="T55"/>
-      <x:c r="U55"/>
-      <x:c r="V55"/>
-      <x:c r="W55"/>
-      <x:c r="X55"/>
-      <x:c r="Y55"/>
-      <x:c r="Z55"/>
+      <x:c r="O55" s="27"/>
+      <x:c r="P55" s="27"/>
+      <x:c r="Q55" s="27"/>
+      <x:c r="R55" s="39"/>
+      <x:c r="S55" s="40"/>
+      <x:c r="T55" s="40"/>
+      <x:c r="U55" s="37"/>
+      <x:c r="V55" s="38"/>
+      <x:c r="W55" s="38"/>
+      <x:c r="X55" s="38"/>
+      <x:c r="Y55" s="37"/>
+      <x:c r="Z55" s="37"/>
+      <x:c r="AA55" s="37"/>
+      <x:c r="AB55" s="37"/>
+      <x:c r="AC55" s="37"/>
     </x:row>
     <x:row r="56" ht="13.550000190734863" customHeight="1">
       <x:c r="A56" s="14"/>
@@ -2596,18 +3097,21 @@
       <x:c r="L56" s="16"/>
       <x:c r="M56" s="16"/>
       <x:c r="N56" s="16"/>
-      <x:c r="O56" s="17"/>
-      <x:c r="P56" s="17"/>
-      <x:c r="Q56" s="15"/>
-      <x:c r="R56" s="14"/>
-      <x:c r="S56"/>
-      <x:c r="T56"/>
-      <x:c r="U56"/>
-      <x:c r="V56"/>
-      <x:c r="W56"/>
-      <x:c r="X56"/>
-      <x:c r="Y56"/>
-      <x:c r="Z56"/>
+      <x:c r="O56" s="27"/>
+      <x:c r="P56" s="27"/>
+      <x:c r="Q56" s="27"/>
+      <x:c r="R56" s="39"/>
+      <x:c r="S56" s="40"/>
+      <x:c r="T56" s="40"/>
+      <x:c r="U56" s="37"/>
+      <x:c r="V56" s="38"/>
+      <x:c r="W56" s="38"/>
+      <x:c r="X56" s="38"/>
+      <x:c r="Y56" s="37"/>
+      <x:c r="Z56" s="37"/>
+      <x:c r="AA56" s="37"/>
+      <x:c r="AB56" s="37"/>
+      <x:c r="AC56" s="37"/>
     </x:row>
     <x:row r="57" ht="13.550000190734863" customHeight="1">
       <x:c r="A57" s="14"/>
@@ -2624,18 +3128,21 @@
       <x:c r="L57" s="16"/>
       <x:c r="M57" s="16"/>
       <x:c r="N57" s="16"/>
-      <x:c r="O57" s="17"/>
-      <x:c r="P57" s="17"/>
-      <x:c r="Q57" s="15"/>
-      <x:c r="R57" s="14"/>
-      <x:c r="S57"/>
-      <x:c r="T57"/>
-      <x:c r="U57"/>
-      <x:c r="V57"/>
-      <x:c r="W57"/>
-      <x:c r="X57"/>
-      <x:c r="Y57"/>
-      <x:c r="Z57"/>
+      <x:c r="O57" s="27"/>
+      <x:c r="P57" s="27"/>
+      <x:c r="Q57" s="27"/>
+      <x:c r="R57" s="39"/>
+      <x:c r="S57" s="40"/>
+      <x:c r="T57" s="40"/>
+      <x:c r="U57" s="37"/>
+      <x:c r="V57" s="38"/>
+      <x:c r="W57" s="38"/>
+      <x:c r="X57" s="38"/>
+      <x:c r="Y57" s="37"/>
+      <x:c r="Z57" s="37"/>
+      <x:c r="AA57" s="37"/>
+      <x:c r="AB57" s="37"/>
+      <x:c r="AC57" s="37"/>
     </x:row>
     <x:row r="58" ht="13.550000190734863" customHeight="1">
       <x:c r="A58" s="14"/>
@@ -2652,18 +3159,21 @@
       <x:c r="L58" s="16"/>
       <x:c r="M58" s="16"/>
       <x:c r="N58" s="16"/>
-      <x:c r="O58" s="17"/>
-      <x:c r="P58" s="17"/>
-      <x:c r="Q58" s="14"/>
-      <x:c r="R58" s="14"/>
-      <x:c r="S58"/>
-      <x:c r="T58"/>
-      <x:c r="U58"/>
-      <x:c r="V58"/>
-      <x:c r="W58"/>
-      <x:c r="X58"/>
-      <x:c r="Y58"/>
-      <x:c r="Z58"/>
+      <x:c r="O58" s="27"/>
+      <x:c r="P58" s="27"/>
+      <x:c r="Q58" s="27"/>
+      <x:c r="R58" s="39"/>
+      <x:c r="S58" s="40"/>
+      <x:c r="T58" s="40"/>
+      <x:c r="U58" s="37"/>
+      <x:c r="V58" s="38"/>
+      <x:c r="W58" s="38"/>
+      <x:c r="X58" s="38"/>
+      <x:c r="Y58" s="37"/>
+      <x:c r="Z58" s="37"/>
+      <x:c r="AA58" s="37"/>
+      <x:c r="AB58" s="37"/>
+      <x:c r="AC58" s="37"/>
     </x:row>
     <x:row r="59" ht="13.550000190734863" customHeight="1">
       <x:c r="A59" s="14"/>
@@ -2680,18 +3190,21 @@
       <x:c r="L59" s="16"/>
       <x:c r="M59" s="16"/>
       <x:c r="N59" s="16"/>
-      <x:c r="O59" s="17"/>
-      <x:c r="P59" s="17"/>
-      <x:c r="Q59" s="15"/>
-      <x:c r="R59" s="15"/>
-      <x:c r="S59"/>
-      <x:c r="T59"/>
-      <x:c r="U59"/>
-      <x:c r="V59"/>
-      <x:c r="W59"/>
-      <x:c r="X59"/>
-      <x:c r="Y59"/>
-      <x:c r="Z59"/>
+      <x:c r="O59" s="27"/>
+      <x:c r="P59" s="27"/>
+      <x:c r="Q59" s="27"/>
+      <x:c r="R59" s="39"/>
+      <x:c r="S59" s="40"/>
+      <x:c r="T59" s="40"/>
+      <x:c r="U59" s="37"/>
+      <x:c r="V59" s="38"/>
+      <x:c r="W59" s="38"/>
+      <x:c r="X59" s="38"/>
+      <x:c r="Y59" s="37"/>
+      <x:c r="Z59" s="37"/>
+      <x:c r="AA59" s="37"/>
+      <x:c r="AB59" s="37"/>
+      <x:c r="AC59" s="37"/>
     </x:row>
     <x:row r="60" ht="13.550000190734863" customHeight="1">
       <x:c r="A60" s="14"/>
@@ -2708,18 +3221,21 @@
       <x:c r="L60" s="16"/>
       <x:c r="M60" s="16"/>
       <x:c r="N60" s="16"/>
-      <x:c r="O60" s="17"/>
-      <x:c r="P60" s="17"/>
-      <x:c r="Q60" s="14"/>
-      <x:c r="R60" s="14"/>
-      <x:c r="S60"/>
-      <x:c r="T60"/>
-      <x:c r="U60"/>
-      <x:c r="V60"/>
-      <x:c r="W60"/>
-      <x:c r="X60"/>
-      <x:c r="Y60"/>
-      <x:c r="Z60"/>
+      <x:c r="O60" s="27"/>
+      <x:c r="P60" s="27"/>
+      <x:c r="Q60" s="27"/>
+      <x:c r="R60" s="39"/>
+      <x:c r="S60" s="40"/>
+      <x:c r="T60" s="40"/>
+      <x:c r="U60" s="37"/>
+      <x:c r="V60" s="38"/>
+      <x:c r="W60" s="38"/>
+      <x:c r="X60" s="38"/>
+      <x:c r="Y60" s="37"/>
+      <x:c r="Z60" s="37"/>
+      <x:c r="AA60" s="37"/>
+      <x:c r="AB60" s="37"/>
+      <x:c r="AC60" s="37"/>
     </x:row>
     <x:row r="61" ht="13.550000190734863" customHeight="1">
       <x:c r="A61" s="14"/>
@@ -2736,18 +3252,21 @@
       <x:c r="L61" s="16"/>
       <x:c r="M61" s="16"/>
       <x:c r="N61" s="16"/>
-      <x:c r="O61" s="17"/>
-      <x:c r="P61" s="17"/>
-      <x:c r="Q61" s="15"/>
-      <x:c r="R61" s="15"/>
-      <x:c r="S61"/>
-      <x:c r="T61"/>
-      <x:c r="U61"/>
-      <x:c r="V61"/>
-      <x:c r="W61"/>
-      <x:c r="X61"/>
-      <x:c r="Y61"/>
-      <x:c r="Z61"/>
+      <x:c r="O61" s="27"/>
+      <x:c r="P61" s="27"/>
+      <x:c r="Q61" s="27"/>
+      <x:c r="R61" s="39"/>
+      <x:c r="S61" s="40"/>
+      <x:c r="T61" s="40"/>
+      <x:c r="U61" s="37"/>
+      <x:c r="V61" s="38"/>
+      <x:c r="W61" s="38"/>
+      <x:c r="X61" s="38"/>
+      <x:c r="Y61" s="37"/>
+      <x:c r="Z61" s="37"/>
+      <x:c r="AA61" s="37"/>
+      <x:c r="AB61" s="37"/>
+      <x:c r="AC61" s="37"/>
     </x:row>
     <x:row r="62" ht="13.550000190734863" customHeight="1">
       <x:c r="A62" s="14"/>
@@ -2764,18 +3283,21 @@
       <x:c r="L62" s="16"/>
       <x:c r="M62" s="16"/>
       <x:c r="N62" s="16"/>
-      <x:c r="O62" s="17"/>
-      <x:c r="P62" s="17"/>
-      <x:c r="Q62" s="15"/>
-      <x:c r="R62" s="15"/>
-      <x:c r="S62"/>
-      <x:c r="T62"/>
-      <x:c r="U62"/>
-      <x:c r="V62"/>
-      <x:c r="W62"/>
-      <x:c r="X62"/>
-      <x:c r="Y62"/>
-      <x:c r="Z62"/>
+      <x:c r="O62" s="27"/>
+      <x:c r="P62" s="27"/>
+      <x:c r="Q62" s="27"/>
+      <x:c r="R62" s="39"/>
+      <x:c r="S62" s="40"/>
+      <x:c r="T62" s="40"/>
+      <x:c r="U62" s="37"/>
+      <x:c r="V62" s="38"/>
+      <x:c r="W62" s="38"/>
+      <x:c r="X62" s="38"/>
+      <x:c r="Y62" s="37"/>
+      <x:c r="Z62" s="37"/>
+      <x:c r="AA62" s="37"/>
+      <x:c r="AB62" s="37"/>
+      <x:c r="AC62" s="37"/>
     </x:row>
     <x:row r="63" ht="13.550000190734863" customHeight="1">
       <x:c r="A63" s="14"/>
@@ -2792,18 +3314,21 @@
       <x:c r="L63" s="16"/>
       <x:c r="M63" s="16"/>
       <x:c r="N63" s="16"/>
-      <x:c r="O63" s="17"/>
-      <x:c r="P63" s="17"/>
-      <x:c r="Q63" s="15"/>
-      <x:c r="R63" s="14"/>
-      <x:c r="S63"/>
-      <x:c r="T63"/>
-      <x:c r="U63"/>
-      <x:c r="V63"/>
-      <x:c r="W63"/>
-      <x:c r="X63"/>
-      <x:c r="Y63"/>
-      <x:c r="Z63"/>
+      <x:c r="O63" s="27"/>
+      <x:c r="P63" s="27"/>
+      <x:c r="Q63" s="27"/>
+      <x:c r="R63" s="39"/>
+      <x:c r="S63" s="40"/>
+      <x:c r="T63" s="40"/>
+      <x:c r="U63" s="37"/>
+      <x:c r="V63" s="38"/>
+      <x:c r="W63" s="38"/>
+      <x:c r="X63" s="38"/>
+      <x:c r="Y63" s="37"/>
+      <x:c r="Z63" s="37"/>
+      <x:c r="AA63" s="37"/>
+      <x:c r="AB63" s="37"/>
+      <x:c r="AC63" s="37"/>
     </x:row>
     <x:row r="64" ht="13.550000190734863" customHeight="1">
       <x:c r="A64" s="14"/>
@@ -2820,18 +3345,21 @@
       <x:c r="L64" s="16"/>
       <x:c r="M64" s="16"/>
       <x:c r="N64" s="16"/>
-      <x:c r="O64" s="17"/>
-      <x:c r="P64" s="17"/>
-      <x:c r="Q64" s="14"/>
-      <x:c r="R64" s="14"/>
-      <x:c r="S64"/>
-      <x:c r="T64"/>
-      <x:c r="U64"/>
-      <x:c r="V64"/>
-      <x:c r="W64"/>
-      <x:c r="X64"/>
-      <x:c r="Y64"/>
-      <x:c r="Z64"/>
+      <x:c r="O64" s="27"/>
+      <x:c r="P64" s="27"/>
+      <x:c r="Q64" s="27"/>
+      <x:c r="R64" s="39"/>
+      <x:c r="S64" s="40"/>
+      <x:c r="T64" s="40"/>
+      <x:c r="U64" s="37"/>
+      <x:c r="V64" s="38"/>
+      <x:c r="W64" s="38"/>
+      <x:c r="X64" s="38"/>
+      <x:c r="Y64" s="37"/>
+      <x:c r="Z64" s="37"/>
+      <x:c r="AA64" s="37"/>
+      <x:c r="AB64" s="37"/>
+      <x:c r="AC64" s="37"/>
     </x:row>
     <x:row r="65" ht="13.550000190734863" customHeight="1">
       <x:c r="A65" s="14"/>
@@ -2848,18 +3376,21 @@
       <x:c r="L65" s="16"/>
       <x:c r="M65" s="16"/>
       <x:c r="N65" s="16"/>
-      <x:c r="O65" s="17"/>
-      <x:c r="P65" s="17"/>
-      <x:c r="Q65" s="15"/>
-      <x:c r="R65" s="15"/>
-      <x:c r="S65"/>
-      <x:c r="T65"/>
-      <x:c r="U65"/>
-      <x:c r="V65"/>
-      <x:c r="W65"/>
-      <x:c r="X65"/>
-      <x:c r="Y65"/>
-      <x:c r="Z65"/>
+      <x:c r="O65" s="27"/>
+      <x:c r="P65" s="27"/>
+      <x:c r="Q65" s="27"/>
+      <x:c r="R65" s="39"/>
+      <x:c r="S65" s="40"/>
+      <x:c r="T65" s="40"/>
+      <x:c r="U65" s="37"/>
+      <x:c r="V65" s="38"/>
+      <x:c r="W65" s="38"/>
+      <x:c r="X65" s="38"/>
+      <x:c r="Y65" s="37"/>
+      <x:c r="Z65" s="37"/>
+      <x:c r="AA65" s="37"/>
+      <x:c r="AB65" s="37"/>
+      <x:c r="AC65" s="37"/>
     </x:row>
     <x:row r="66" ht="13.550000190734863" customHeight="1">
       <x:c r="A66" s="14"/>
@@ -2876,18 +3407,21 @@
       <x:c r="L66" s="16"/>
       <x:c r="M66" s="16"/>
       <x:c r="N66" s="16"/>
-      <x:c r="O66" s="17"/>
-      <x:c r="P66" s="17"/>
-      <x:c r="Q66" s="15"/>
-      <x:c r="R66" s="15"/>
-      <x:c r="S66"/>
-      <x:c r="T66"/>
-      <x:c r="U66"/>
-      <x:c r="V66"/>
-      <x:c r="W66"/>
-      <x:c r="X66"/>
-      <x:c r="Y66"/>
-      <x:c r="Z66"/>
+      <x:c r="O66" s="27"/>
+      <x:c r="P66" s="27"/>
+      <x:c r="Q66" s="27"/>
+      <x:c r="R66" s="39"/>
+      <x:c r="S66" s="40"/>
+      <x:c r="T66" s="40"/>
+      <x:c r="U66" s="37"/>
+      <x:c r="V66" s="38"/>
+      <x:c r="W66" s="38"/>
+      <x:c r="X66" s="38"/>
+      <x:c r="Y66" s="37"/>
+      <x:c r="Z66" s="37"/>
+      <x:c r="AA66" s="37"/>
+      <x:c r="AB66" s="37"/>
+      <x:c r="AC66" s="37"/>
     </x:row>
     <x:row r="67" ht="13.550000190734863" customHeight="1">
       <x:c r="A67" s="14"/>
@@ -2904,18 +3438,21 @@
       <x:c r="L67" s="16"/>
       <x:c r="M67" s="16"/>
       <x:c r="N67" s="16"/>
-      <x:c r="O67" s="17"/>
-      <x:c r="P67" s="17"/>
-      <x:c r="Q67" s="15"/>
-      <x:c r="R67" s="15"/>
-      <x:c r="S67"/>
-      <x:c r="T67"/>
-      <x:c r="U67"/>
-      <x:c r="V67"/>
-      <x:c r="W67"/>
-      <x:c r="X67"/>
-      <x:c r="Y67"/>
-      <x:c r="Z67"/>
+      <x:c r="O67" s="27"/>
+      <x:c r="P67" s="27"/>
+      <x:c r="Q67" s="27"/>
+      <x:c r="R67" s="39"/>
+      <x:c r="S67" s="40"/>
+      <x:c r="T67" s="40"/>
+      <x:c r="U67" s="37"/>
+      <x:c r="V67" s="38"/>
+      <x:c r="W67" s="38"/>
+      <x:c r="X67" s="38"/>
+      <x:c r="Y67" s="37"/>
+      <x:c r="Z67" s="37"/>
+      <x:c r="AA67" s="37"/>
+      <x:c r="AB67" s="37"/>
+      <x:c r="AC67" s="37"/>
     </x:row>
     <x:row r="68" ht="13.550000190734863" customHeight="1">
       <x:c r="A68" s="14"/>
@@ -2932,18 +3469,21 @@
       <x:c r="L68" s="16"/>
       <x:c r="M68" s="16"/>
       <x:c r="N68" s="16"/>
-      <x:c r="O68" s="17"/>
-      <x:c r="P68" s="17"/>
-      <x:c r="Q68" s="15"/>
-      <x:c r="R68" s="14"/>
-      <x:c r="S68"/>
-      <x:c r="T68"/>
-      <x:c r="U68"/>
-      <x:c r="V68"/>
-      <x:c r="W68"/>
-      <x:c r="X68"/>
-      <x:c r="Y68"/>
-      <x:c r="Z68"/>
+      <x:c r="O68" s="27"/>
+      <x:c r="P68" s="27"/>
+      <x:c r="Q68" s="27"/>
+      <x:c r="R68" s="39"/>
+      <x:c r="S68" s="40"/>
+      <x:c r="T68" s="40"/>
+      <x:c r="U68" s="37"/>
+      <x:c r="V68" s="38"/>
+      <x:c r="W68" s="38"/>
+      <x:c r="X68" s="38"/>
+      <x:c r="Y68" s="37"/>
+      <x:c r="Z68" s="37"/>
+      <x:c r="AA68" s="37"/>
+      <x:c r="AB68" s="37"/>
+      <x:c r="AC68" s="37"/>
     </x:row>
     <x:row r="69" ht="13.550000190734863" customHeight="1">
       <x:c r="A69" s="14"/>
@@ -2960,18 +3500,21 @@
       <x:c r="L69" s="16"/>
       <x:c r="M69" s="16"/>
       <x:c r="N69" s="16"/>
-      <x:c r="O69" s="17"/>
-      <x:c r="P69" s="17"/>
-      <x:c r="Q69" s="14"/>
-      <x:c r="R69" s="14"/>
-      <x:c r="S69"/>
-      <x:c r="T69"/>
-      <x:c r="U69"/>
-      <x:c r="V69"/>
-      <x:c r="W69"/>
-      <x:c r="X69"/>
-      <x:c r="Y69"/>
-      <x:c r="Z69"/>
+      <x:c r="O69" s="27"/>
+      <x:c r="P69" s="27"/>
+      <x:c r="Q69" s="27"/>
+      <x:c r="R69" s="39"/>
+      <x:c r="S69" s="40"/>
+      <x:c r="T69" s="40"/>
+      <x:c r="U69" s="37"/>
+      <x:c r="V69" s="38"/>
+      <x:c r="W69" s="38"/>
+      <x:c r="X69" s="38"/>
+      <x:c r="Y69" s="37"/>
+      <x:c r="Z69" s="37"/>
+      <x:c r="AA69" s="37"/>
+      <x:c r="AB69" s="37"/>
+      <x:c r="AC69" s="37"/>
     </x:row>
     <x:row r="70" ht="13.550000190734863" customHeight="1">
       <x:c r="A70" s="14"/>
@@ -2988,18 +3531,21 @@
       <x:c r="L70" s="16"/>
       <x:c r="M70" s="16"/>
       <x:c r="N70" s="16"/>
-      <x:c r="O70" s="17"/>
-      <x:c r="P70" s="17"/>
-      <x:c r="Q70" s="15"/>
-      <x:c r="R70" s="15"/>
-      <x:c r="S70"/>
-      <x:c r="T70"/>
-      <x:c r="U70"/>
-      <x:c r="V70"/>
-      <x:c r="W70"/>
-      <x:c r="X70"/>
-      <x:c r="Y70"/>
-      <x:c r="Z70"/>
+      <x:c r="O70" s="27"/>
+      <x:c r="P70" s="27"/>
+      <x:c r="Q70" s="27"/>
+      <x:c r="R70" s="39"/>
+      <x:c r="S70" s="40"/>
+      <x:c r="T70" s="40"/>
+      <x:c r="U70" s="37"/>
+      <x:c r="V70" s="38"/>
+      <x:c r="W70" s="38"/>
+      <x:c r="X70" s="38"/>
+      <x:c r="Y70" s="37"/>
+      <x:c r="Z70" s="37"/>
+      <x:c r="AA70" s="37"/>
+      <x:c r="AB70" s="37"/>
+      <x:c r="AC70" s="37"/>
     </x:row>
     <x:row r="71" ht="13.550000190734863" customHeight="1">
       <x:c r="A71" s="14"/>
@@ -3016,18 +3562,21 @@
       <x:c r="L71" s="16"/>
       <x:c r="M71" s="16"/>
       <x:c r="N71" s="16"/>
-      <x:c r="O71" s="17"/>
-      <x:c r="P71" s="17"/>
-      <x:c r="Q71" s="14"/>
-      <x:c r="R71" s="14"/>
-      <x:c r="S71"/>
-      <x:c r="T71"/>
-      <x:c r="U71"/>
-      <x:c r="V71"/>
-      <x:c r="W71"/>
-      <x:c r="X71"/>
-      <x:c r="Y71"/>
-      <x:c r="Z71"/>
+      <x:c r="O71" s="27"/>
+      <x:c r="P71" s="27"/>
+      <x:c r="Q71" s="27"/>
+      <x:c r="R71" s="39"/>
+      <x:c r="S71" s="40"/>
+      <x:c r="T71" s="40"/>
+      <x:c r="U71" s="37"/>
+      <x:c r="V71" s="38"/>
+      <x:c r="W71" s="38"/>
+      <x:c r="X71" s="38"/>
+      <x:c r="Y71" s="37"/>
+      <x:c r="Z71" s="37"/>
+      <x:c r="AA71" s="37"/>
+      <x:c r="AB71" s="37"/>
+      <x:c r="AC71" s="37"/>
     </x:row>
     <x:row r="72" ht="13.550000190734863" customHeight="1">
       <x:c r="A72" s="14"/>
@@ -3044,18 +3593,21 @@
       <x:c r="L72" s="16"/>
       <x:c r="M72" s="16"/>
       <x:c r="N72" s="16"/>
-      <x:c r="O72" s="17"/>
-      <x:c r="P72" s="17"/>
-      <x:c r="Q72" s="15"/>
-      <x:c r="R72" s="15"/>
-      <x:c r="S72"/>
-      <x:c r="T72"/>
-      <x:c r="U72"/>
-      <x:c r="V72"/>
-      <x:c r="W72"/>
-      <x:c r="X72"/>
-      <x:c r="Y72"/>
-      <x:c r="Z72"/>
+      <x:c r="O72" s="27"/>
+      <x:c r="P72" s="27"/>
+      <x:c r="Q72" s="27"/>
+      <x:c r="R72" s="39"/>
+      <x:c r="S72" s="40"/>
+      <x:c r="T72" s="40"/>
+      <x:c r="U72" s="37"/>
+      <x:c r="V72" s="38"/>
+      <x:c r="W72" s="38"/>
+      <x:c r="X72" s="38"/>
+      <x:c r="Y72" s="37"/>
+      <x:c r="Z72" s="37"/>
+      <x:c r="AA72" s="37"/>
+      <x:c r="AB72" s="37"/>
+      <x:c r="AC72" s="37"/>
     </x:row>
     <x:row r="73" ht="13.550000190734863" customHeight="1">
       <x:c r="A73" s="14"/>
@@ -3072,18 +3624,21 @@
       <x:c r="L73" s="16"/>
       <x:c r="M73" s="16"/>
       <x:c r="N73" s="16"/>
-      <x:c r="O73" s="17"/>
-      <x:c r="P73" s="17"/>
-      <x:c r="Q73" s="15"/>
-      <x:c r="R73" s="15"/>
-      <x:c r="S73"/>
-      <x:c r="T73"/>
-      <x:c r="U73"/>
-      <x:c r="V73"/>
-      <x:c r="W73"/>
-      <x:c r="X73"/>
-      <x:c r="Y73"/>
-      <x:c r="Z73"/>
+      <x:c r="O73" s="27"/>
+      <x:c r="P73" s="27"/>
+      <x:c r="Q73" s="27"/>
+      <x:c r="R73" s="39"/>
+      <x:c r="S73" s="40"/>
+      <x:c r="T73" s="40"/>
+      <x:c r="U73" s="37"/>
+      <x:c r="V73" s="38"/>
+      <x:c r="W73" s="38"/>
+      <x:c r="X73" s="38"/>
+      <x:c r="Y73" s="37"/>
+      <x:c r="Z73" s="37"/>
+      <x:c r="AA73" s="37"/>
+      <x:c r="AB73" s="37"/>
+      <x:c r="AC73" s="37"/>
     </x:row>
     <x:row r="74" ht="13.550000190734863" customHeight="1">
       <x:c r="A74" s="14"/>
@@ -3100,18 +3655,21 @@
       <x:c r="L74" s="16"/>
       <x:c r="M74" s="16"/>
       <x:c r="N74" s="16"/>
-      <x:c r="O74" s="17"/>
-      <x:c r="P74" s="17"/>
-      <x:c r="Q74" s="15"/>
-      <x:c r="R74" s="14"/>
-      <x:c r="S74"/>
-      <x:c r="T74"/>
-      <x:c r="U74"/>
-      <x:c r="V74"/>
-      <x:c r="W74"/>
-      <x:c r="X74"/>
-      <x:c r="Y74"/>
-      <x:c r="Z74"/>
+      <x:c r="O74" s="27"/>
+      <x:c r="P74" s="27"/>
+      <x:c r="Q74" s="27"/>
+      <x:c r="R74" s="39"/>
+      <x:c r="S74" s="40"/>
+      <x:c r="T74" s="40"/>
+      <x:c r="U74" s="37"/>
+      <x:c r="V74" s="38"/>
+      <x:c r="W74" s="38"/>
+      <x:c r="X74" s="38"/>
+      <x:c r="Y74" s="37"/>
+      <x:c r="Z74" s="37"/>
+      <x:c r="AA74" s="37"/>
+      <x:c r="AB74" s="37"/>
+      <x:c r="AC74" s="37"/>
     </x:row>
     <x:row r="75" ht="13.550000190734863" customHeight="1">
       <x:c r="A75" s="14"/>
@@ -3128,18 +3686,21 @@
       <x:c r="L75" s="16"/>
       <x:c r="M75" s="16"/>
       <x:c r="N75" s="16"/>
-      <x:c r="O75" s="17"/>
-      <x:c r="P75" s="17"/>
-      <x:c r="Q75" s="15"/>
-      <x:c r="R75" s="15"/>
-      <x:c r="S75"/>
-      <x:c r="T75"/>
-      <x:c r="U75"/>
-      <x:c r="V75"/>
-      <x:c r="W75"/>
-      <x:c r="X75"/>
-      <x:c r="Y75"/>
-      <x:c r="Z75"/>
+      <x:c r="O75" s="27"/>
+      <x:c r="P75" s="27"/>
+      <x:c r="Q75" s="27"/>
+      <x:c r="R75" s="39"/>
+      <x:c r="S75" s="40"/>
+      <x:c r="T75" s="40"/>
+      <x:c r="U75" s="37"/>
+      <x:c r="V75" s="38"/>
+      <x:c r="W75" s="38"/>
+      <x:c r="X75" s="38"/>
+      <x:c r="Y75" s="37"/>
+      <x:c r="Z75" s="37"/>
+      <x:c r="AA75" s="37"/>
+      <x:c r="AB75" s="37"/>
+      <x:c r="AC75" s="37"/>
     </x:row>
     <x:row r="76" ht="13.550000190734863" customHeight="1">
       <x:c r="A76" s="14"/>
@@ -3156,18 +3717,21 @@
       <x:c r="L76" s="16"/>
       <x:c r="M76" s="16"/>
       <x:c r="N76" s="16"/>
-      <x:c r="O76" s="17"/>
-      <x:c r="P76" s="17"/>
-      <x:c r="Q76" s="15"/>
-      <x:c r="R76" s="14"/>
-      <x:c r="S76"/>
-      <x:c r="T76"/>
-      <x:c r="U76"/>
-      <x:c r="V76"/>
-      <x:c r="W76"/>
-      <x:c r="X76"/>
-      <x:c r="Y76"/>
-      <x:c r="Z76"/>
+      <x:c r="O76" s="27"/>
+      <x:c r="P76" s="27"/>
+      <x:c r="Q76" s="27"/>
+      <x:c r="R76" s="39"/>
+      <x:c r="S76" s="40"/>
+      <x:c r="T76" s="40"/>
+      <x:c r="U76" s="37"/>
+      <x:c r="V76" s="38"/>
+      <x:c r="W76" s="38"/>
+      <x:c r="X76" s="38"/>
+      <x:c r="Y76" s="37"/>
+      <x:c r="Z76" s="37"/>
+      <x:c r="AA76" s="37"/>
+      <x:c r="AB76" s="37"/>
+      <x:c r="AC76" s="37"/>
     </x:row>
     <x:row r="77" ht="13.550000190734863" customHeight="1">
       <x:c r="A77" s="14"/>
@@ -3184,18 +3748,21 @@
       <x:c r="L77" s="16"/>
       <x:c r="M77" s="16"/>
       <x:c r="N77" s="16"/>
-      <x:c r="O77" s="17"/>
-      <x:c r="P77" s="17"/>
-      <x:c r="Q77" s="15"/>
-      <x:c r="R77" s="15"/>
-      <x:c r="S77"/>
-      <x:c r="T77"/>
-      <x:c r="U77"/>
-      <x:c r="V77"/>
-      <x:c r="W77"/>
-      <x:c r="X77"/>
-      <x:c r="Y77"/>
-      <x:c r="Z77"/>
+      <x:c r="O77" s="27"/>
+      <x:c r="P77" s="27"/>
+      <x:c r="Q77" s="27"/>
+      <x:c r="R77" s="39"/>
+      <x:c r="S77" s="40"/>
+      <x:c r="T77" s="40"/>
+      <x:c r="U77" s="37"/>
+      <x:c r="V77" s="38"/>
+      <x:c r="W77" s="38"/>
+      <x:c r="X77" s="38"/>
+      <x:c r="Y77" s="37"/>
+      <x:c r="Z77" s="37"/>
+      <x:c r="AA77" s="37"/>
+      <x:c r="AB77" s="37"/>
+      <x:c r="AC77" s="37"/>
     </x:row>
     <x:row r="78" ht="13.550000190734863" customHeight="1">
       <x:c r="A78" s="14"/>
@@ -3212,18 +3779,21 @@
       <x:c r="L78" s="16"/>
       <x:c r="M78" s="16"/>
       <x:c r="N78" s="16"/>
-      <x:c r="O78" s="17"/>
-      <x:c r="P78" s="17"/>
-      <x:c r="Q78" s="15"/>
-      <x:c r="R78" s="15"/>
-      <x:c r="S78"/>
-      <x:c r="T78"/>
-      <x:c r="U78"/>
-      <x:c r="V78"/>
-      <x:c r="W78"/>
-      <x:c r="X78"/>
-      <x:c r="Y78"/>
-      <x:c r="Z78"/>
+      <x:c r="O78" s="27"/>
+      <x:c r="P78" s="27"/>
+      <x:c r="Q78" s="27"/>
+      <x:c r="R78" s="39"/>
+      <x:c r="S78" s="40"/>
+      <x:c r="T78" s="40"/>
+      <x:c r="U78" s="37"/>
+      <x:c r="V78" s="38"/>
+      <x:c r="W78" s="38"/>
+      <x:c r="X78" s="38"/>
+      <x:c r="Y78" s="37"/>
+      <x:c r="Z78" s="37"/>
+      <x:c r="AA78" s="37"/>
+      <x:c r="AB78" s="37"/>
+      <x:c r="AC78" s="37"/>
     </x:row>
     <x:row r="79" ht="13.550000190734863" customHeight="1">
       <x:c r="A79" s="14"/>
@@ -3240,18 +3810,21 @@
       <x:c r="L79" s="16"/>
       <x:c r="M79" s="16"/>
       <x:c r="N79" s="16"/>
-      <x:c r="O79" s="17"/>
-      <x:c r="P79" s="17"/>
-      <x:c r="Q79" s="15"/>
-      <x:c r="R79" s="15"/>
-      <x:c r="S79"/>
-      <x:c r="T79"/>
-      <x:c r="U79"/>
-      <x:c r="V79"/>
-      <x:c r="W79"/>
-      <x:c r="X79"/>
-      <x:c r="Y79"/>
-      <x:c r="Z79"/>
+      <x:c r="O79" s="27"/>
+      <x:c r="P79" s="27"/>
+      <x:c r="Q79" s="27"/>
+      <x:c r="R79" s="39"/>
+      <x:c r="S79" s="40"/>
+      <x:c r="T79" s="40"/>
+      <x:c r="U79" s="37"/>
+      <x:c r="V79" s="38"/>
+      <x:c r="W79" s="38"/>
+      <x:c r="X79" s="38"/>
+      <x:c r="Y79" s="37"/>
+      <x:c r="Z79" s="37"/>
+      <x:c r="AA79" s="37"/>
+      <x:c r="AB79" s="37"/>
+      <x:c r="AC79" s="37"/>
     </x:row>
     <x:row r="80" ht="13.550000190734863" customHeight="1">
       <x:c r="A80" s="14"/>
@@ -3268,18 +3841,21 @@
       <x:c r="L80" s="16"/>
       <x:c r="M80" s="16"/>
       <x:c r="N80" s="16"/>
-      <x:c r="O80" s="17"/>
-      <x:c r="P80" s="17"/>
-      <x:c r="Q80" s="15"/>
-      <x:c r="R80" s="14"/>
-      <x:c r="S80"/>
-      <x:c r="T80"/>
-      <x:c r="U80"/>
-      <x:c r="V80"/>
-      <x:c r="W80"/>
-      <x:c r="X80"/>
-      <x:c r="Y80"/>
-      <x:c r="Z80"/>
+      <x:c r="O80" s="27"/>
+      <x:c r="P80" s="27"/>
+      <x:c r="Q80" s="27"/>
+      <x:c r="R80" s="39"/>
+      <x:c r="S80" s="40"/>
+      <x:c r="T80" s="40"/>
+      <x:c r="U80" s="37"/>
+      <x:c r="V80" s="38"/>
+      <x:c r="W80" s="38"/>
+      <x:c r="X80" s="38"/>
+      <x:c r="Y80" s="37"/>
+      <x:c r="Z80" s="37"/>
+      <x:c r="AA80" s="37"/>
+      <x:c r="AB80" s="37"/>
+      <x:c r="AC80" s="37"/>
     </x:row>
     <x:row r="81" ht="13.550000190734863" customHeight="1">
       <x:c r="A81" s="14"/>
@@ -3296,18 +3872,21 @@
       <x:c r="L81" s="16"/>
       <x:c r="M81" s="16"/>
       <x:c r="N81" s="16"/>
-      <x:c r="O81" s="17"/>
-      <x:c r="P81" s="17"/>
-      <x:c r="Q81" s="15"/>
-      <x:c r="R81" s="15"/>
-      <x:c r="S81"/>
-      <x:c r="T81"/>
-      <x:c r="U81"/>
-      <x:c r="V81"/>
-      <x:c r="W81"/>
-      <x:c r="X81"/>
-      <x:c r="Y81"/>
-      <x:c r="Z81"/>
+      <x:c r="O81" s="27"/>
+      <x:c r="P81" s="27"/>
+      <x:c r="Q81" s="27"/>
+      <x:c r="R81" s="39"/>
+      <x:c r="S81" s="40"/>
+      <x:c r="T81" s="40"/>
+      <x:c r="U81" s="37"/>
+      <x:c r="V81" s="38"/>
+      <x:c r="W81" s="38"/>
+      <x:c r="X81" s="38"/>
+      <x:c r="Y81" s="37"/>
+      <x:c r="Z81" s="37"/>
+      <x:c r="AA81" s="37"/>
+      <x:c r="AB81" s="37"/>
+      <x:c r="AC81" s="37"/>
     </x:row>
     <x:row r="82" ht="13.550000190734863" customHeight="1">
       <x:c r="A82" s="14"/>
@@ -3324,18 +3903,21 @@
       <x:c r="L82" s="16"/>
       <x:c r="M82" s="16"/>
       <x:c r="N82" s="16"/>
-      <x:c r="O82" s="17"/>
-      <x:c r="P82" s="17"/>
-      <x:c r="Q82" s="15"/>
-      <x:c r="R82" s="15"/>
-      <x:c r="S82"/>
-      <x:c r="T82"/>
-      <x:c r="U82"/>
-      <x:c r="V82"/>
-      <x:c r="W82"/>
-      <x:c r="X82"/>
-      <x:c r="Y82"/>
-      <x:c r="Z82"/>
+      <x:c r="O82" s="27"/>
+      <x:c r="P82" s="27"/>
+      <x:c r="Q82" s="27"/>
+      <x:c r="R82" s="39"/>
+      <x:c r="S82" s="40"/>
+      <x:c r="T82" s="40"/>
+      <x:c r="U82" s="37"/>
+      <x:c r="V82" s="38"/>
+      <x:c r="W82" s="38"/>
+      <x:c r="X82" s="38"/>
+      <x:c r="Y82" s="37"/>
+      <x:c r="Z82" s="37"/>
+      <x:c r="AA82" s="37"/>
+      <x:c r="AB82" s="37"/>
+      <x:c r="AC82" s="37"/>
     </x:row>
     <x:row r="83" ht="13.550000190734863" customHeight="1">
       <x:c r="A83" s="14"/>
@@ -3352,18 +3934,21 @@
       <x:c r="L83" s="16"/>
       <x:c r="M83" s="16"/>
       <x:c r="N83" s="16"/>
-      <x:c r="O83" s="17"/>
-      <x:c r="P83" s="17"/>
-      <x:c r="Q83" s="15"/>
-      <x:c r="R83" s="14"/>
-      <x:c r="S83"/>
-      <x:c r="T83"/>
-      <x:c r="U83"/>
-      <x:c r="V83"/>
-      <x:c r="W83"/>
-      <x:c r="X83"/>
-      <x:c r="Y83"/>
-      <x:c r="Z83"/>
+      <x:c r="O83" s="27"/>
+      <x:c r="P83" s="27"/>
+      <x:c r="Q83" s="27"/>
+      <x:c r="R83" s="39"/>
+      <x:c r="S83" s="40"/>
+      <x:c r="T83" s="40"/>
+      <x:c r="U83" s="37"/>
+      <x:c r="V83" s="38"/>
+      <x:c r="W83" s="38"/>
+      <x:c r="X83" s="38"/>
+      <x:c r="Y83" s="37"/>
+      <x:c r="Z83" s="37"/>
+      <x:c r="AA83" s="37"/>
+      <x:c r="AB83" s="37"/>
+      <x:c r="AC83" s="37"/>
     </x:row>
     <x:row r="84" ht="13.550000190734863" customHeight="1">
       <x:c r="A84" s="14"/>
@@ -3380,18 +3965,21 @@
       <x:c r="L84" s="16"/>
       <x:c r="M84" s="16"/>
       <x:c r="N84" s="16"/>
-      <x:c r="O84" s="17"/>
-      <x:c r="P84" s="17"/>
-      <x:c r="Q84" s="15"/>
-      <x:c r="R84" s="15"/>
-      <x:c r="S84"/>
-      <x:c r="T84"/>
-      <x:c r="U84"/>
-      <x:c r="V84"/>
-      <x:c r="W84"/>
-      <x:c r="X84"/>
-      <x:c r="Y84"/>
-      <x:c r="Z84"/>
+      <x:c r="O84" s="27"/>
+      <x:c r="P84" s="27"/>
+      <x:c r="Q84" s="27"/>
+      <x:c r="R84" s="39"/>
+      <x:c r="S84" s="40"/>
+      <x:c r="T84" s="40"/>
+      <x:c r="U84" s="37"/>
+      <x:c r="V84" s="38"/>
+      <x:c r="W84" s="38"/>
+      <x:c r="X84" s="38"/>
+      <x:c r="Y84" s="37"/>
+      <x:c r="Z84" s="37"/>
+      <x:c r="AA84" s="37"/>
+      <x:c r="AB84" s="37"/>
+      <x:c r="AC84" s="37"/>
     </x:row>
     <x:row r="85" ht="13.550000190734863" customHeight="1">
       <x:c r="A85" s="14"/>
@@ -3408,18 +3996,21 @@
       <x:c r="L85" s="16"/>
       <x:c r="M85" s="16"/>
       <x:c r="N85" s="16"/>
-      <x:c r="O85" s="17"/>
-      <x:c r="P85" s="17"/>
-      <x:c r="Q85" s="15"/>
-      <x:c r="R85" s="15"/>
-      <x:c r="S85"/>
-      <x:c r="T85"/>
-      <x:c r="U85"/>
-      <x:c r="V85"/>
-      <x:c r="W85"/>
-      <x:c r="X85"/>
-      <x:c r="Y85"/>
-      <x:c r="Z85"/>
+      <x:c r="O85" s="27"/>
+      <x:c r="P85" s="27"/>
+      <x:c r="Q85" s="27"/>
+      <x:c r="R85" s="39"/>
+      <x:c r="S85" s="40"/>
+      <x:c r="T85" s="40"/>
+      <x:c r="U85" s="37"/>
+      <x:c r="V85" s="38"/>
+      <x:c r="W85" s="38"/>
+      <x:c r="X85" s="38"/>
+      <x:c r="Y85" s="37"/>
+      <x:c r="Z85" s="37"/>
+      <x:c r="AA85" s="37"/>
+      <x:c r="AB85" s="37"/>
+      <x:c r="AC85" s="37"/>
     </x:row>
     <x:row r="86" ht="13.550000190734863" customHeight="1">
       <x:c r="A86" s="14"/>
@@ -3436,18 +4027,21 @@
       <x:c r="L86" s="16"/>
       <x:c r="M86" s="16"/>
       <x:c r="N86" s="16"/>
-      <x:c r="O86" s="17"/>
-      <x:c r="P86" s="17"/>
-      <x:c r="Q86" s="15"/>
-      <x:c r="R86" s="15"/>
-      <x:c r="S86"/>
-      <x:c r="T86"/>
-      <x:c r="U86"/>
-      <x:c r="V86"/>
-      <x:c r="W86"/>
-      <x:c r="X86"/>
-      <x:c r="Y86"/>
-      <x:c r="Z86"/>
+      <x:c r="O86" s="27"/>
+      <x:c r="P86" s="27"/>
+      <x:c r="Q86" s="27"/>
+      <x:c r="R86" s="39"/>
+      <x:c r="S86" s="40"/>
+      <x:c r="T86" s="40"/>
+      <x:c r="U86" s="37"/>
+      <x:c r="V86" s="38"/>
+      <x:c r="W86" s="38"/>
+      <x:c r="X86" s="38"/>
+      <x:c r="Y86" s="37"/>
+      <x:c r="Z86" s="37"/>
+      <x:c r="AA86" s="37"/>
+      <x:c r="AB86" s="37"/>
+      <x:c r="AC86" s="37"/>
     </x:row>
     <x:row r="87" ht="13.550000190734863" customHeight="1">
       <x:c r="A87" s="14"/>
@@ -3464,18 +4058,21 @@
       <x:c r="L87" s="16"/>
       <x:c r="M87" s="16"/>
       <x:c r="N87" s="16"/>
-      <x:c r="O87" s="17"/>
-      <x:c r="P87" s="17"/>
-      <x:c r="Q87" s="15"/>
-      <x:c r="R87" s="15"/>
-      <x:c r="S87"/>
-      <x:c r="T87"/>
-      <x:c r="U87"/>
-      <x:c r="V87"/>
-      <x:c r="W87"/>
-      <x:c r="X87"/>
-      <x:c r="Y87"/>
-      <x:c r="Z87"/>
+      <x:c r="O87" s="27"/>
+      <x:c r="P87" s="27"/>
+      <x:c r="Q87" s="27"/>
+      <x:c r="R87" s="39"/>
+      <x:c r="S87" s="40"/>
+      <x:c r="T87" s="40"/>
+      <x:c r="U87" s="37"/>
+      <x:c r="V87" s="38"/>
+      <x:c r="W87" s="38"/>
+      <x:c r="X87" s="38"/>
+      <x:c r="Y87" s="37"/>
+      <x:c r="Z87" s="37"/>
+      <x:c r="AA87" s="37"/>
+      <x:c r="AB87" s="37"/>
+      <x:c r="AC87" s="37"/>
     </x:row>
     <x:row r="88" ht="13.550000190734863" customHeight="1">
       <x:c r="A88" s="14"/>
@@ -3492,18 +4089,21 @@
       <x:c r="L88" s="16"/>
       <x:c r="M88" s="16"/>
       <x:c r="N88" s="16"/>
-      <x:c r="O88" s="17"/>
-      <x:c r="P88" s="17"/>
-      <x:c r="Q88" s="15"/>
-      <x:c r="R88" s="15"/>
-      <x:c r="S88"/>
-      <x:c r="T88"/>
-      <x:c r="U88"/>
-      <x:c r="V88"/>
-      <x:c r="W88"/>
-      <x:c r="X88"/>
-      <x:c r="Y88"/>
-      <x:c r="Z88"/>
+      <x:c r="O88" s="27"/>
+      <x:c r="P88" s="27"/>
+      <x:c r="Q88" s="27"/>
+      <x:c r="R88" s="39"/>
+      <x:c r="S88" s="40"/>
+      <x:c r="T88" s="40"/>
+      <x:c r="U88" s="37"/>
+      <x:c r="V88" s="38"/>
+      <x:c r="W88" s="38"/>
+      <x:c r="X88" s="38"/>
+      <x:c r="Y88" s="37"/>
+      <x:c r="Z88" s="37"/>
+      <x:c r="AA88" s="37"/>
+      <x:c r="AB88" s="37"/>
+      <x:c r="AC88" s="37"/>
     </x:row>
     <x:row r="89" ht="13.550000190734863" customHeight="1">
       <x:c r="A89" s="14"/>
@@ -3520,18 +4120,21 @@
       <x:c r="L89" s="16"/>
       <x:c r="M89" s="16"/>
       <x:c r="N89" s="16"/>
-      <x:c r="O89" s="17"/>
-      <x:c r="P89" s="17"/>
-      <x:c r="Q89" s="15"/>
-      <x:c r="R89" s="15"/>
-      <x:c r="S89"/>
-      <x:c r="T89"/>
-      <x:c r="U89"/>
-      <x:c r="V89"/>
-      <x:c r="W89"/>
-      <x:c r="X89"/>
-      <x:c r="Y89"/>
-      <x:c r="Z89"/>
+      <x:c r="O89" s="27"/>
+      <x:c r="P89" s="27"/>
+      <x:c r="Q89" s="27"/>
+      <x:c r="R89" s="39"/>
+      <x:c r="S89" s="40"/>
+      <x:c r="T89" s="40"/>
+      <x:c r="U89" s="37"/>
+      <x:c r="V89" s="38"/>
+      <x:c r="W89" s="38"/>
+      <x:c r="X89" s="38"/>
+      <x:c r="Y89" s="37"/>
+      <x:c r="Z89" s="37"/>
+      <x:c r="AA89" s="37"/>
+      <x:c r="AB89" s="37"/>
+      <x:c r="AC89" s="37"/>
     </x:row>
     <x:row r="90" ht="13.550000190734863" customHeight="1">
       <x:c r="A90" s="14"/>
@@ -3548,18 +4151,21 @@
       <x:c r="L90" s="16"/>
       <x:c r="M90" s="16"/>
       <x:c r="N90" s="16"/>
-      <x:c r="O90" s="17"/>
-      <x:c r="P90" s="17"/>
-      <x:c r="Q90" s="15"/>
-      <x:c r="R90" s="15"/>
-      <x:c r="S90"/>
-      <x:c r="T90"/>
-      <x:c r="U90"/>
-      <x:c r="V90"/>
-      <x:c r="W90"/>
-      <x:c r="X90"/>
-      <x:c r="Y90"/>
-      <x:c r="Z90"/>
+      <x:c r="O90" s="27"/>
+      <x:c r="P90" s="27"/>
+      <x:c r="Q90" s="27"/>
+      <x:c r="R90" s="39"/>
+      <x:c r="S90" s="40"/>
+      <x:c r="T90" s="40"/>
+      <x:c r="U90" s="37"/>
+      <x:c r="V90" s="38"/>
+      <x:c r="W90" s="38"/>
+      <x:c r="X90" s="38"/>
+      <x:c r="Y90" s="37"/>
+      <x:c r="Z90" s="37"/>
+      <x:c r="AA90" s="37"/>
+      <x:c r="AB90" s="37"/>
+      <x:c r="AC90" s="37"/>
     </x:row>
     <x:row r="91" ht="13.550000190734863" customHeight="1">
       <x:c r="A91" s="14"/>
@@ -3576,18 +4182,21 @@
       <x:c r="L91" s="16"/>
       <x:c r="M91" s="16"/>
       <x:c r="N91" s="16"/>
-      <x:c r="O91" s="17"/>
-      <x:c r="P91" s="17"/>
-      <x:c r="Q91" s="15"/>
-      <x:c r="R91" s="15"/>
-      <x:c r="S91"/>
-      <x:c r="T91"/>
-      <x:c r="U91"/>
-      <x:c r="V91"/>
-      <x:c r="W91"/>
-      <x:c r="X91"/>
-      <x:c r="Y91"/>
-      <x:c r="Z91"/>
+      <x:c r="O91" s="27"/>
+      <x:c r="P91" s="27"/>
+      <x:c r="Q91" s="27"/>
+      <x:c r="R91" s="39"/>
+      <x:c r="S91" s="40"/>
+      <x:c r="T91" s="40"/>
+      <x:c r="U91" s="37"/>
+      <x:c r="V91" s="38"/>
+      <x:c r="W91" s="38"/>
+      <x:c r="X91" s="38"/>
+      <x:c r="Y91" s="37"/>
+      <x:c r="Z91" s="37"/>
+      <x:c r="AA91" s="37"/>
+      <x:c r="AB91" s="37"/>
+      <x:c r="AC91" s="37"/>
     </x:row>
     <x:row r="92" ht="13.550000190734863" customHeight="1">
       <x:c r="A92" s="14"/>
@@ -3604,18 +4213,21 @@
       <x:c r="L92" s="16"/>
       <x:c r="M92" s="16"/>
       <x:c r="N92" s="16"/>
-      <x:c r="O92" s="17"/>
-      <x:c r="P92" s="17"/>
-      <x:c r="Q92" s="15"/>
-      <x:c r="R92" s="15"/>
-      <x:c r="S92"/>
-      <x:c r="T92"/>
-      <x:c r="U92"/>
-      <x:c r="V92"/>
-      <x:c r="W92"/>
-      <x:c r="X92"/>
-      <x:c r="Y92"/>
-      <x:c r="Z92"/>
+      <x:c r="O92" s="27"/>
+      <x:c r="P92" s="27"/>
+      <x:c r="Q92" s="27"/>
+      <x:c r="R92" s="39"/>
+      <x:c r="S92" s="40"/>
+      <x:c r="T92" s="40"/>
+      <x:c r="U92" s="37"/>
+      <x:c r="V92" s="38"/>
+      <x:c r="W92" s="38"/>
+      <x:c r="X92" s="38"/>
+      <x:c r="Y92" s="37"/>
+      <x:c r="Z92" s="37"/>
+      <x:c r="AA92" s="37"/>
+      <x:c r="AB92" s="37"/>
+      <x:c r="AC92" s="37"/>
     </x:row>
     <x:row r="93" ht="13.550000190734863" customHeight="1">
       <x:c r="A93" s="14"/>
@@ -3632,18 +4244,21 @@
       <x:c r="L93" s="16"/>
       <x:c r="M93" s="16"/>
       <x:c r="N93" s="16"/>
-      <x:c r="O93" s="17"/>
-      <x:c r="P93" s="17"/>
-      <x:c r="Q93" s="15"/>
-      <x:c r="R93" s="15"/>
-      <x:c r="S93"/>
-      <x:c r="T93"/>
-      <x:c r="U93"/>
-      <x:c r="V93"/>
-      <x:c r="W93"/>
-      <x:c r="X93"/>
-      <x:c r="Y93"/>
-      <x:c r="Z93"/>
+      <x:c r="O93" s="27"/>
+      <x:c r="P93" s="27"/>
+      <x:c r="Q93" s="27"/>
+      <x:c r="R93" s="39"/>
+      <x:c r="S93" s="40"/>
+      <x:c r="T93" s="40"/>
+      <x:c r="U93" s="37"/>
+      <x:c r="V93" s="38"/>
+      <x:c r="W93" s="38"/>
+      <x:c r="X93" s="38"/>
+      <x:c r="Y93" s="37"/>
+      <x:c r="Z93" s="37"/>
+      <x:c r="AA93" s="37"/>
+      <x:c r="AB93" s="37"/>
+      <x:c r="AC93" s="37"/>
     </x:row>
     <x:row r="94" ht="13.550000190734863" customHeight="1">
       <x:c r="A94" s="14"/>
@@ -3660,18 +4275,21 @@
       <x:c r="L94" s="16"/>
       <x:c r="M94" s="16"/>
       <x:c r="N94" s="16"/>
-      <x:c r="O94" s="17"/>
-      <x:c r="P94" s="17"/>
-      <x:c r="Q94" s="15"/>
-      <x:c r="R94" s="15"/>
-      <x:c r="S94"/>
-      <x:c r="T94"/>
-      <x:c r="U94"/>
-      <x:c r="V94"/>
-      <x:c r="W94"/>
-      <x:c r="X94"/>
-      <x:c r="Y94"/>
-      <x:c r="Z94"/>
+      <x:c r="O94" s="27"/>
+      <x:c r="P94" s="27"/>
+      <x:c r="Q94" s="27"/>
+      <x:c r="R94" s="39"/>
+      <x:c r="S94" s="40"/>
+      <x:c r="T94" s="40"/>
+      <x:c r="U94" s="37"/>
+      <x:c r="V94" s="38"/>
+      <x:c r="W94" s="38"/>
+      <x:c r="X94" s="38"/>
+      <x:c r="Y94" s="37"/>
+      <x:c r="Z94" s="37"/>
+      <x:c r="AA94" s="37"/>
+      <x:c r="AB94" s="37"/>
+      <x:c r="AC94" s="37"/>
     </x:row>
     <x:row r="95" ht="13.550000190734863" customHeight="1">
       <x:c r="A95" s="14"/>
@@ -3688,18 +4306,21 @@
       <x:c r="L95" s="16"/>
       <x:c r="M95" s="16"/>
       <x:c r="N95" s="16"/>
-      <x:c r="O95" s="17"/>
-      <x:c r="P95" s="17"/>
-      <x:c r="Q95" s="15"/>
-      <x:c r="R95" s="15"/>
-      <x:c r="S95"/>
-      <x:c r="T95"/>
-      <x:c r="U95"/>
-      <x:c r="V95"/>
-      <x:c r="W95"/>
-      <x:c r="X95"/>
-      <x:c r="Y95"/>
-      <x:c r="Z95"/>
+      <x:c r="O95" s="27"/>
+      <x:c r="P95" s="27"/>
+      <x:c r="Q95" s="27"/>
+      <x:c r="R95" s="39"/>
+      <x:c r="S95" s="40"/>
+      <x:c r="T95" s="40"/>
+      <x:c r="U95" s="37"/>
+      <x:c r="V95" s="38"/>
+      <x:c r="W95" s="38"/>
+      <x:c r="X95" s="38"/>
+      <x:c r="Y95" s="37"/>
+      <x:c r="Z95" s="37"/>
+      <x:c r="AA95" s="37"/>
+      <x:c r="AB95" s="37"/>
+      <x:c r="AC95" s="37"/>
     </x:row>
     <x:row r="96" ht="13.550000190734863" customHeight="1">
       <x:c r="A96" s="14"/>
@@ -3716,18 +4337,21 @@
       <x:c r="L96" s="16"/>
       <x:c r="M96" s="16"/>
       <x:c r="N96" s="16"/>
-      <x:c r="O96" s="17"/>
-      <x:c r="P96" s="17"/>
-      <x:c r="Q96" s="15"/>
-      <x:c r="R96" s="15"/>
-      <x:c r="S96"/>
-      <x:c r="T96"/>
-      <x:c r="U96"/>
-      <x:c r="V96"/>
-      <x:c r="W96"/>
-      <x:c r="X96"/>
-      <x:c r="Y96"/>
-      <x:c r="Z96"/>
+      <x:c r="O96" s="27"/>
+      <x:c r="P96" s="27"/>
+      <x:c r="Q96" s="27"/>
+      <x:c r="R96" s="39"/>
+      <x:c r="S96" s="40"/>
+      <x:c r="T96" s="40"/>
+      <x:c r="U96" s="37"/>
+      <x:c r="V96" s="38"/>
+      <x:c r="W96" s="38"/>
+      <x:c r="X96" s="38"/>
+      <x:c r="Y96" s="37"/>
+      <x:c r="Z96" s="37"/>
+      <x:c r="AA96" s="37"/>
+      <x:c r="AB96" s="37"/>
+      <x:c r="AC96" s="37"/>
     </x:row>
     <x:row r="97" ht="13.550000190734863" customHeight="1">
       <x:c r="A97" s="14"/>
@@ -3744,18 +4368,21 @@
       <x:c r="L97" s="16"/>
       <x:c r="M97" s="16"/>
       <x:c r="N97" s="16"/>
-      <x:c r="O97" s="17"/>
-      <x:c r="P97" s="17"/>
-      <x:c r="Q97" s="15"/>
-      <x:c r="R97" s="15"/>
-      <x:c r="S97"/>
-      <x:c r="T97"/>
-      <x:c r="U97"/>
-      <x:c r="V97"/>
-      <x:c r="W97"/>
-      <x:c r="X97"/>
-      <x:c r="Y97"/>
-      <x:c r="Z97"/>
+      <x:c r="O97" s="27"/>
+      <x:c r="P97" s="27"/>
+      <x:c r="Q97" s="27"/>
+      <x:c r="R97" s="39"/>
+      <x:c r="S97" s="40"/>
+      <x:c r="T97" s="40"/>
+      <x:c r="U97" s="37"/>
+      <x:c r="V97" s="38"/>
+      <x:c r="W97" s="38"/>
+      <x:c r="X97" s="38"/>
+      <x:c r="Y97" s="37"/>
+      <x:c r="Z97" s="37"/>
+      <x:c r="AA97" s="37"/>
+      <x:c r="AB97" s="37"/>
+      <x:c r="AC97" s="37"/>
     </x:row>
     <x:row r="98" ht="13.550000190734863" customHeight="1">
       <x:c r="A98" s="14"/>
@@ -3772,18 +4399,21 @@
       <x:c r="L98" s="16"/>
       <x:c r="M98" s="16"/>
       <x:c r="N98" s="16"/>
-      <x:c r="O98" s="17"/>
-      <x:c r="P98" s="17"/>
-      <x:c r="Q98" s="15"/>
-      <x:c r="R98" s="15"/>
-      <x:c r="S98"/>
-      <x:c r="T98"/>
-      <x:c r="U98"/>
-      <x:c r="V98"/>
-      <x:c r="W98"/>
-      <x:c r="X98"/>
-      <x:c r="Y98"/>
-      <x:c r="Z98"/>
+      <x:c r="O98" s="27"/>
+      <x:c r="P98" s="27"/>
+      <x:c r="Q98" s="27"/>
+      <x:c r="R98" s="39"/>
+      <x:c r="S98" s="40"/>
+      <x:c r="T98" s="40"/>
+      <x:c r="U98" s="37"/>
+      <x:c r="V98" s="38"/>
+      <x:c r="W98" s="38"/>
+      <x:c r="X98" s="38"/>
+      <x:c r="Y98" s="37"/>
+      <x:c r="Z98" s="37"/>
+      <x:c r="AA98" s="37"/>
+      <x:c r="AB98" s="37"/>
+      <x:c r="AC98" s="37"/>
     </x:row>
     <x:row r="99" ht="13.550000190734863" customHeight="1">
       <x:c r="A99" s="14"/>
@@ -3800,18 +4430,21 @@
       <x:c r="L99" s="16"/>
       <x:c r="M99" s="16"/>
       <x:c r="N99" s="16"/>
-      <x:c r="O99" s="17"/>
-      <x:c r="P99" s="17"/>
-      <x:c r="Q99" s="15"/>
-      <x:c r="R99" s="15"/>
-      <x:c r="S99"/>
-      <x:c r="T99"/>
-      <x:c r="U99"/>
-      <x:c r="V99"/>
-      <x:c r="W99"/>
-      <x:c r="X99"/>
-      <x:c r="Y99"/>
-      <x:c r="Z99"/>
+      <x:c r="O99" s="27"/>
+      <x:c r="P99" s="27"/>
+      <x:c r="Q99" s="27"/>
+      <x:c r="R99" s="39"/>
+      <x:c r="S99" s="40"/>
+      <x:c r="T99" s="40"/>
+      <x:c r="U99" s="37"/>
+      <x:c r="V99" s="38"/>
+      <x:c r="W99" s="38"/>
+      <x:c r="X99" s="38"/>
+      <x:c r="Y99" s="37"/>
+      <x:c r="Z99" s="37"/>
+      <x:c r="AA99" s="37"/>
+      <x:c r="AB99" s="37"/>
+      <x:c r="AC99" s="37"/>
     </x:row>
     <x:row r="100" ht="13.550000190734863" customHeight="1">
       <x:c r="A100" s="14"/>
@@ -3828,18 +4461,21 @@
       <x:c r="L100" s="16"/>
       <x:c r="M100" s="16"/>
       <x:c r="N100" s="16"/>
-      <x:c r="O100" s="17"/>
-      <x:c r="P100" s="17"/>
-      <x:c r="Q100" s="15"/>
-      <x:c r="R100" s="15"/>
-      <x:c r="S100"/>
-      <x:c r="T100"/>
-      <x:c r="U100"/>
-      <x:c r="V100"/>
-      <x:c r="W100"/>
-      <x:c r="X100"/>
-      <x:c r="Y100"/>
-      <x:c r="Z100"/>
+      <x:c r="O100" s="27"/>
+      <x:c r="P100" s="27"/>
+      <x:c r="Q100" s="27"/>
+      <x:c r="R100" s="39"/>
+      <x:c r="S100" s="40"/>
+      <x:c r="T100" s="40"/>
+      <x:c r="U100" s="37"/>
+      <x:c r="V100" s="38"/>
+      <x:c r="W100" s="38"/>
+      <x:c r="X100" s="38"/>
+      <x:c r="Y100" s="37"/>
+      <x:c r="Z100" s="37"/>
+      <x:c r="AA100" s="37"/>
+      <x:c r="AB100" s="37"/>
+      <x:c r="AC100" s="37"/>
     </x:row>
     <x:row r="101" ht="13.550000190734863" customHeight="1">
       <x:c r="A101" s="14"/>
@@ -3856,18 +4492,21 @@
       <x:c r="L101" s="16"/>
       <x:c r="M101" s="16"/>
       <x:c r="N101" s="16"/>
-      <x:c r="O101" s="17"/>
-      <x:c r="P101" s="17"/>
-      <x:c r="Q101" s="15"/>
-      <x:c r="R101" s="15"/>
-      <x:c r="S101"/>
-      <x:c r="T101"/>
-      <x:c r="U101"/>
-      <x:c r="V101"/>
-      <x:c r="W101"/>
-      <x:c r="X101"/>
-      <x:c r="Y101"/>
-      <x:c r="Z101"/>
+      <x:c r="O101" s="27"/>
+      <x:c r="P101" s="27"/>
+      <x:c r="Q101" s="27"/>
+      <x:c r="R101" s="39"/>
+      <x:c r="S101" s="40"/>
+      <x:c r="T101" s="40"/>
+      <x:c r="U101" s="37"/>
+      <x:c r="V101" s="38"/>
+      <x:c r="W101" s="38"/>
+      <x:c r="X101" s="38"/>
+      <x:c r="Y101" s="37"/>
+      <x:c r="Z101" s="37"/>
+      <x:c r="AA101" s="37"/>
+      <x:c r="AB101" s="37"/>
+      <x:c r="AC101" s="37"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>